<commit_message>
fix(inputs): P1-02 rename phase-1 sheet History to Request_History
Excel reserves the sheet name History and ExcelJS (the seed's reader) refuses a
workbook that has one. Renamed in scripts/inputs_p1 and validate_inputs.py and
regenerated docs/inputs/BCS_inputs_p1.xlsx (same data, deterministic).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/inputs/BCS_inputs_p1.xlsx
+++ b/docs/inputs/BCS_inputs_p1.xlsx
@@ -31,7 +31,7 @@
     <sheet name="Settings" sheetId="22" state="visible" r:id="rId22"/>
     <sheet name="WHT_Types" sheetId="23" state="visible" r:id="rId23"/>
     <sheet name="CompanyBankAccounts" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="History" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="Request_History" sheetId="25" state="visible" r:id="rId25"/>
     <sheet name="DocSamples" sheetId="26" state="visible" r:id="rId26"/>
     <sheet name="Scenarios" sheetId="27" state="visible" r:id="rId27"/>
   </sheets>
@@ -764,7 +764,7 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>History</t>
+          <t>Request_History</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1988,7 +1988,7 @@
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>กุญแจงบที่ไม่มีปี (คำขอใน History อ้างคอลัมน์นี้)</t>
+          <t>กุญแจงบที่ไม่มีปี (คำขอใน Request_History อ้างคอลัมน์นี้)</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
@@ -64707,7 +64707,7 @@
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="42" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
@@ -64848,7 +64848,7 @@
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>คำขอใน History</t>
+          <t>คำขอใน Request_History</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
@@ -69848,7 +69848,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>History · pattern ESCALATED</t>
+          <t>Request_History · pattern ESCALATED</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -69875,7 +69875,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>History · eqp_02 FUL-001</t>
+          <t>Request_History · eqp_02 FUL-001</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -69902,7 +69902,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>History · pattern SPLIT</t>
+          <t>Request_History · pattern SPLIT</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -69929,7 +69929,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>History · pattern DUPLICATE</t>
+          <t>Request_History · pattern DUPLICATE</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -69956,7 +69956,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>History · pattern RENEWAL</t>
+          <t>Request_History · pattern RENEWAL</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -69983,7 +69983,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>History · pattern OVERDUE</t>
+          <t>Request_History · pattern OVERDUE</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -70010,7 +70010,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>History · pattern LOW_BUDGET · Budget MKT-OPEX</t>
+          <t>Request_History · pattern LOW_BUDGET · Budget MKT-OPEX</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -70145,7 +70145,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>History · invoiceScenario</t>
+          <t>Request_History · invoiceScenario</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -70172,7 +70172,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>History · paymentStatus</t>
+          <t>Request_History · paymentStatus</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -70199,7 +70199,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>WHT_Types · History whtIncomeType</t>
+          <t>WHT_Types · Request_History whtIncomeType</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -70226,7 +70226,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>History · form processesPersonalData = Y</t>
+          <t>Request_History · form processesPersonalData = Y</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -70253,7 +70253,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>History · gross &gt; 100,000</t>
+          <t>Request_History · gross &gt; 100,000</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -70307,7 +70307,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>History · pattern OVERDUE (pm_p07) · Workflow_Reviewers RV-03 ถึง RV-05</t>
+          <t>Request_History · pattern OVERDUE (pm_p07) · Workflow_Reviewers RV-03 ถึง RV-05</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -73558,7 +73558,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>คำขอซื้อต่อเดือนโดยประมาณ (ชีต History สร้างด้วยอัตรานี้)</t>
+          <t>คำขอซื้อต่อเดือนโดยประมาณ (ชีต Request_History สร้างด้วยอัตรานี้)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">

</xml_diff>

<commit_message>
docs(spec): P1-04 checklists of S6 S8 S9 S13 S17, P1-07 base, OQ and ADR
- §16.14 to §16.18: checklist and effort table of each step (99 items), from
  the sub-specs in docs/sub-specs
- §16.13 P1-07 rewritten as the shared base the lanes rely on (new DOA types,
  subject registry, central step-up, AI-assist contract, reserved sections)
- §18.1 ADR-067..070 (base, main numbers) and lane ranges 101-110, 121-134,
  141-148, 161-167, each with docs/decisions/ADR-nnn.md and an index row
- §18.3 OQ-40 and lane ranges 101-116, 121-137, 141-148, 161-171; every OQ
  has a question in the phase-1 workbook (p1_texts.py, make.py rebuilt it)
- sub-specs point to the spec for checklists and OQ instead of keeping copies

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/inputs/BCS_inputs_p1.xlsx
+++ b/docs/inputs/BCS_inputs_p1.xlsx
@@ -70354,7 +70354,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I72"/>
+  <dimension ref="A1:I108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -70363,7 +70363,7 @@
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="41" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="35" customWidth="1" min="7" max="7"/>
     <col width="27" customWidth="1" min="8" max="8"/>
     <col width="41" customWidth="1" min="9" max="9"/>
   </cols>
@@ -72013,7 +72013,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>FR-WF-101</t>
+          <t>OQ-101 FR-WF-101</t>
         </is>
       </c>
     </row>
@@ -72050,7 +72050,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>FR-WF-102</t>
+          <t>OQ-102 FR-WF-102</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -72087,12 +72087,12 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>ร่างในชีต DOA_P1_Draft (OVER_BUDGET)</t>
+          <t>ข้อ OB-01 ถึง OB-03 ในชีต DOA ฉบับ 1</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>FR-BUD-101</t>
+          <t>OQ-104 OQ-40 FR-BUD-101</t>
         </is>
       </c>
     </row>
@@ -72124,12 +72124,12 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>ร่างในชีต DOA_P1_Draft (BUDGET_TRANSFER)</t>
+          <t>ข้อ BT-01 ถึง BT-03 ในชีต DOA ฉบับ 1</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>FR-BUD-103</t>
+          <t>OQ-105 OQ-40 FR-BUD-103</t>
         </is>
       </c>
     </row>
@@ -72166,7 +72166,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>FR-BUD-102</t>
+          <t>OQ-106 FR-BUD-102</t>
         </is>
       </c>
     </row>
@@ -72203,7 +72203,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>FR-INT-103</t>
+          <t>OQ-103 FR-INT-103</t>
         </is>
       </c>
     </row>
@@ -72277,12 +72277,12 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>ราคา 1% หรือ 1,000 บาท · จำนวน 0%</t>
+          <t>ราคาเกินได้ไม่เกิน 1% และไม่เกิน 1,000 บาทต่อบรรทัด (ต้องผ่านทั้งคู่) · จำนวน 0% · ส่วนเกินในเกณฑ์ใช้งบเพิ่มเอง · ตั้งค่าโดย BCS จากคำตอบ</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>BR-MATCH-02</t>
+          <t>OQ-121 BR-MATCH-02</t>
         </is>
       </c>
     </row>
@@ -72319,7 +72319,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>FR-AP-101</t>
+          <t>OQ-124 FR-AP-101</t>
         </is>
       </c>
     </row>
@@ -72356,7 +72356,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>BR-WHT-01</t>
+          <t>OQ-122 BR-WHT-01</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -72393,12 +72393,12 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>ระบบออก 50 ทวิ และไฟล์ ภ.ง.ด. ตามรูปแบบกรมสรรพากร</t>
+          <t>demo: 50 ทวิ ที่ผู้ทำบัญชีต้องตรวจรูปแบบ และไฟล์สรุปแบบกลางที่ไม่ใช่รูปแบบยื่น · รูปแบบยื่นจริงรอตัวอย่าง</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>BR-WHT-02</t>
+          <t>OQ-123 BR-WHT-02</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -72435,12 +72435,12 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>หัก 5% คืนเมื่อพ้นประกัน</t>
+          <t>หัก 5% ของยอดก่อน VAT คืนหลังพ้นประกัน 365 วัน</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>FR-AP-106</t>
+          <t>OQ-125 FR-AP-106</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -72477,12 +72477,12 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>ร่างในชีต DOA_P1_Draft (PO_CHANGE)</t>
+          <t>ข้อ PC-01 PC-02 ในชีต DOA ฉบับ 1</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>FR-AP-107</t>
+          <t>OQ-126 OQ-40 FR-AP-107</t>
         </is>
       </c>
     </row>
@@ -72519,7 +72519,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>FR-PAY-101</t>
+          <t>OQ-130 FR-PAY-101</t>
         </is>
       </c>
     </row>
@@ -72551,12 +72551,12 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>ร่างในชีต DOA_P1_Draft (PAYMENT_RUN)</t>
+          <t>ข้อ PAY-01 PAY-02 ในชีต DOA ฉบับ 1</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>FR-PAY-101</t>
+          <t>OQ-131 OQ-40 FR-PAY-101 BR-SOD-04</t>
         </is>
       </c>
     </row>
@@ -72593,7 +72593,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>P0-03</t>
+          <t>P0-03 FR-PAY-102</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -72630,12 +72630,12 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>ร่างในชีต DOA_P1_Draft (BANK_ACCOUNT_CHANGE)</t>
+          <t>ข้อ BA-01 ในชีต DOA ฉบับ 1</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>FR-PAY-102</t>
+          <t>OQ-133 OQ-40 FR-PAY-102 BR-SOD-05</t>
         </is>
       </c>
     </row>
@@ -72672,7 +72672,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>FR-PAY-103</t>
+          <t>OQ-134 FR-PAY-103</t>
         </is>
       </c>
     </row>
@@ -72709,7 +72709,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>§12</t>
+          <t>OQ-144 §12</t>
         </is>
       </c>
     </row>
@@ -72788,7 +72788,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>§12.4</t>
+          <t>OQ-142 §12.4</t>
         </is>
       </c>
     </row>
@@ -72825,7 +72825,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>FR-PLT-301</t>
+          <t>OQ-166 FR-PLT-301</t>
         </is>
       </c>
     </row>
@@ -72862,7 +72862,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>FR-PLT-301</t>
+          <t>OQ-163 FR-PLT-301</t>
         </is>
       </c>
     </row>
@@ -72899,266 +72899,1618 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>FR-LINE-301</t>
+          <t>OQ-161 FR-LINE-301</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>B-01</t>
+          <t>Q-64</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>BCS</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>ทีม BCS</t>
+          <t>CEO COO กฎหมาย DPO</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>LIFF ใช้ LINE MINI App หรือ LINE Login channel ใน production</t>
+          <t>การ์ดอนุมัติใน LINE และการแจ้งเตือน (push) บนหน้าจอล็อกของแอป ควรแสดงข้อมูลราคาและสรุปจาก AI ได้แค่ไหน (ตัวเลขเต็มอยู่ในหน้างานที่ยืนยันตัวตนแล้ว)</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>การเผยแพร่และการ login ใน LINE</t>
+          <t>ข้อมูลที่ค้างในแชทหรือเห็นได้บนหน้าจอล็อก เทียบกับความสะดวกของผู้อนุมัติ</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>MINI App + ตรวจ ID token เอง</t>
+          <t>การ์ด LINE มีข้อมูลเดิม + ป้ายราคาแบบรวมไม่ระบุรายการ (เช่น ราคาสูงกว่าค่ากลางย้อนหลัง 1 รายการ สูงสุด +8%) ไม่มีราคาต่อหน่วยและสรุป AI · push มีชนิดงานและเลขเอกสารเท่านั้น</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>OQ-16</t>
+          <t>OQ-107 FR-DOA-101 FR-AI-301 FR-PLT-301 BR-NOTI-01</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>B-02</t>
+          <t>Q-65</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>BCS</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>ทีม BCS</t>
+          <t>จัดซื้อ ตรวจสอบภายใน</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>วิธีสร้าง PDF</t>
+          <t>ใครควรเห็นแผงราคาอ้างอิง (ราคาที่เคยซื้อจาก PO ย้อนหลังทั้งองค์กร) นอกจากผู้อนุมัติและผู้ตรวจของคำขอนั้น</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>คุณภาพภาษาไทยบนเอกสาร</t>
+          <t>ราคาซื้อย้อนหลังเป็นข้อมูลภายในของจัดซื้อ</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>ตัดสินแล้ว (ADR-044)</t>
+          <t>ผู้ได้รับงานของคำขอนั้นและผู้มีสิทธิ์ดู PO ทั้งองค์กร · ผู้ขอ ผู้ติดตาม และหัวหน้าฝ่ายที่ไม่ได้รับงานไม่เห็น</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>OQ-18</t>
+          <t>OQ-116 FR-DOA-101</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>B-03</t>
+          <t>Q-66</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>BCS</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>ทีม BCS</t>
+          <t>IT ตรวจสอบภายใน</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>ยืนยันการประกาศพระราชกฤษฎีกาคง VAT 7%</t>
+          <t>ต้องการระบบทดลอง (UAT) แยกสำหรับลองตั้งค่าก่อนใช้จริงไหม ใครตั้งต้นระบบทดลอง และใครเป็นคนย้ายค่าที่ทดลองแล้วเข้าระบบจริง</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>อัตรา VAT ในระบบ</t>
+          <t>ลดความเสี่ยงตอนเปลี่ยนการตั้งค่า</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>7% และให้ PLATFORM_ADMIN ยืนยัน</t>
+          <t>องค์กรทดลองคู่แฝดในระบบเดียวกัน คนของบริษัทตั้งต้นเอง ไม่คัดลอกข้อมูลจริง ผัง หรือ DOA · นำเข้าเป็นร่างแล้วอนุมัติตามปกติ</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>OQ-29</t>
+          <t>OQ-108 FR-PLT-101</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>B-04</t>
+          <t>Q-67</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>BCS</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>ทีม BCS</t>
+          <t>CEO CFO</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>ปิดโมดูลขณะมีเอกสารค้าง</t>
+          <t>ให้ผู้ดูแล DOA (เช่น ฝ่ายการเงินหรือเลขานุการบริษัท) แยกจากผู้ดูแลระบบไหม และใครเป็นคนแต่งตั้ง</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>การเปลี่ยนแพ็กเกจ</t>
+          <t>การแยกหน้าที่ของผู้ร่าง DOA</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>ปฏิเสธและแสดงรายการเอกสาร</t>
+          <t>มีบทบาทผู้ดูแล DOA · ผู้ดูแลระบบยังร่างได้จนกว่าจะเปิดการแยกผ่าน DOA ฉบับใหม่ · ห้ามแต่งตั้งตัวเอง</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>OQ-33</t>
+          <t>OQ-109 OQ-34 FR-ADM-101</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>B-05</t>
+          <t>Q-68</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>BCS</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>ทีม BCS</t>
+          <t>CEO ตรวจสอบภายใน</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>ผู้ให้บริการอีเมล hosting และที่เก็บไฟล์ของ production</t>
+          <t>การเปลี่ยนกฎผู้ตรวจคู่ขนาน (เพิ่มหรือตัดฝ่ายที่ต้องตรวจ) ต้องให้ใครอนุมัติ</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>ต้นทุนและที่ตั้งข้อมูล</t>
+          <t>การตัดผู้ตรวจออกทำให้การควบคุมอ่อนลง</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>ยังไม่ตัดสิน</t>
+          <t>ผู้อนุมัติการแก้ DOA (กรรมการผู้จัดการ) พร้อมยืนยันตัวตนทุกครั้ง (PIN หรือ passkey) บนเว็บ</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>ADR-031 ADR-032 ADR-033</t>
+          <t>OQ-110 FR-WF-103</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>B-06</t>
+          <t>Q-69</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>BCS</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>ทีม BCS</t>
+          <t>CEO COO</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>ราคาและแพ็กเกจที่จะเสนอหลัง demo ระยะ 1</t>
+          <t>เมื่อเปลี่ยนผู้ดำรงตำแหน่งหรือย้ายฝ่าย เอกสารที่ยังรอขั้นถัดไปหรือรออยู่ ควรไปหาผู้ดำรงตำแหน่งคนใหม่ใช่ไหม</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>สัญญาและขอบเขต</t>
+          <t>งานไม่ค้างที่คนที่พ้นตำแหน่งแล้ว</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>ตามขนาดองค์กรและโมดูล</t>
+          <t>ไปหาผู้ดำรงคนปัจจุบัน ณ เวลาที่ถึงขั้นนั้น โดยใช้ DOA ฉบับเดิม</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>ADR-009</t>
+          <t>OQ-111 FR-WF-104</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
+          <t>Q-70</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>กฎหมาย DPO</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>QR บนใบขอซื้อและใบสั่งซื้อ คนที่สแกนโดยไม่ login (เช่น ผู้ขาย) ควรเห็นข้อมูลอะไร</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>ตรวจเอกสารจริงได้โดยไม่เปิดเผยข้อมูลเกินจำเป็น</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>เลขที่ ชนิด สถานะล่าสุด วันที่ และชื่อบริษัท · ไม่แสดงยอดเงินและชื่อคน</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>OQ-112 FR-DOA-102</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Q-71</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>บัญชี งบประมาณ</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>ควรเตือนการใช้งบที่กี่ % ให้คาดการณ์ว่าจะใช้เกินงบตั้งแต่เมื่อไร และส่งถึงใคร</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>เตือนก่อนงบหมด</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>เตือนที่ 80% และ 100% · คาดการณ์เมื่อผ่านปีงบไป 30 วันขึ้นไป · ผู้จัดการฝ่ายและผู้ดูแลงบในสรุปรายวัน</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>OQ-113 FR-BUD-104</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Q-72</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>จัดซื้อ</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>สินค้าที่มีราคาตกลงรายปีแล้ว ผู้ขอแก้ราคาหรือเลือกผู้ขายรายอื่นได้ไหม และยังต้องมีใบเสนอราคา 3 รายไหม</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>ราคาตกลงถูกใช้จริงและการควบคุมใบเสนอราคา</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>ล็อกราคาตกลง · เลือกรายอื่นได้เมื่อกรอกเหตุผล · ยังใช้กฎใบเสนอราคา 3 รายเดิม</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>OQ-114 FR-INT-102 BR-FORM-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Q-73</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>ตรวจสอบภายใน</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>การแก้ฟอร์มที่เปลี่ยนกฎเอกสารแนบ (เช่น เกณฑ์ใบเสนอราคา 3 ราย หรือ DPA) ต้องมีคนอนุมัติไหม</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>การควบคุมเอกสารประกอบการซื้อ</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>ผู้ดูแลระบบเผยแพร่ได้และแจ้งผู้ตรวจสอบทันที (เหมือนเดิม)</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>OQ-115 FR-INT-104</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Q-74</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>บัญชี</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>VAT ในใบแจ้งหนี้ต่างจากที่ระบบคำนวณเกิน 1 บาท หรือผู้ขายที่ไม่จด VAT เรียกเก็บ VAT ให้ระบบหยุดใบนั้นไว้จนบัญชีแก้หรือปฏิเสธใช่ไหม</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>ภาษีซื้อที่ขอคืนได้และยอดจ่าย</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>หยุดเป็นรายการไม่ตรง (ชั้น 1 เดิมแค่เตือน)</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>OQ-121 BR-VAT-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Q-75</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>บัญชี</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>เงินได้ต่ำกว่า 1,000 บาทไม่หักภาษี ณ ที่จ่าย ให้นับต่อการจ่ายแต่ละครั้งหรือรวมทั้ง PO งานที่หักเงินประกันผลงาน หักภาษีส่วนประกันตอนคืนใช่ไหม และภาษีปัดเศษต่อใบหรือต่อการจ่าย</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>ยอดภาษีที่หักและยอดโอน</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>นับรวมต่อ PO · หักภาษีส่วนประกันตอนคืน · ปัดครั้งเดียวต่อประเภทในแต่ละการจ่าย</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>OQ-122 BR-WHT-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Q-76</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>กฎหมาย DPO บัญชี</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>เลขบัตรประชาชนของผู้รับเหมาบุคคลธรรมดาบน 50 ทวิ และใบแนบ ภ.ง.ด.3 ให้ใครเห็นเลขเต็มได้บ้าง และทะเบียนผู้ขายที่ฝ่ายจัดซื้อเห็นเลขเต็มอยู่แล้วต้องปิดด้วยไหม</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>ข้อมูลส่วนบุคคล (PDPA)</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>FINANCE ที่ได้สิทธิ์ดูเลขเต็มเท่านั้น และบันทึกทุกการเปิด · ทะเบียนผู้ขายปรับก่อน go-live</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>OQ-123 BR-WHT-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Q-77</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>IT บัญชี</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>ตั้ง forward อีเมลจากกล่องรับใบแจ้งหนี้ของฝ่ายบัญชีไปยังที่อยู่ที่ BCS สร้างให้ได้ไหม หรือต้องให้ระบบอ่านกล่องอีเมลของบริษัทเอง</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>รับใบแจ้งหนี้อัตโนมัติ</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>forward ไปที่อยู่เฉพาะของบริษัทใน BCS</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>OQ-124 FR-AP-101</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Q-78</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>CFO ตรวจสอบภายใน</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>ใบแจ้งหนี้ราคาสูงกว่า PO เกินเกณฑ์ ใครอนุมัติส่วนต่าง วงเงินเท่าไร นับรวม VAT ไหม และคนบันทึกใบแจ้งหนี้ห้ามเป็นผู้สั่งซื้อหรือผู้ตรวจรับของ PO นั้นใช่ไหม</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>อำนาจอนุมัติส่วนต่างและการแบ่งแยกหน้าที่</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>ข้อ IE ในชีต DOA ฉบับ 1 (INVOICE_EXCEPTION) · นับตามฐาน DOA · ห้ามคนเดียวกัน</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>OQ-127 OQ-40 FR-AP-105</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Q-79</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>บัญชี</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>ให้ระบบเสนอรหัสบัญชีจากใบแจ้งหนี้ของผู้ขายและหมวดสินค้าเดียวกันใน 365 วันก่อนให้คนยืนยันได้ไหม และ cost center ยึดตามบรรทัดงบใช่ไหม</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>รหัสบัญชีในไฟล์ส่ง Express</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>ประวัติ 365 วัน แล้วรหัสของบรรทัดงบ · cost center ตามบรรทัดงบ แก้ได้พร้อมเหตุผล</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>OQ-128 FR-AP-108</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>ผังบัญชีส่วนที่ใช้กับการซื้อ</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Q-80</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>บัญชี การเงิน</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>ใบแจ้งหนี้หนึ่งใบรวมหลาย PO ไหม มีใบลดหนี้หรือใบเพิ่มหนี้บ่อยแค่ไหน และนับเครดิตจากวันที่ใบแจ้งหนี้หรือวันวางบิล</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>ขอบเขตใบแจ้งหนี้และวันครบกำหนดจ่าย</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>หนึ่งใบต่อหนึ่ง PO · ระยะ 1 ไม่รับใบลดหนี้ · นับจากวันที่ใบแจ้งหนี้</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>OQ-129 FR-AP-101</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>ตัวอย่างใบลดหนี้และใบวางบิล</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Q-81</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>การเงิน ตรวจสอบภายใน</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>ผู้ขายที่เลิกกิจการ ออกจากระบบ VAT หรือไม่พบในทะเบียน ยังจ่ายเงินในรอบจ่ายได้ไหม (บล็อกหรือเตือน) และบัญชีที่เพิ่งเปลี่ยนนับกี่วัน</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>ธงในรอบจ่ายที่ผู้อนุมัติต้องเห็นก่อนอนุมัติ</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>เตือนและให้ผู้เตรียมใส่เหตุผล ไม่บล็อก · 30 วัน</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>OQ-132 FR-PAY-101 BR-SUP-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Q-82</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>การเงิน</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>ธนาคารส่งไฟล์ผลการโอนกลับมาไหม รูปแบบใด และอยากให้นำเข้าระบบแทนการบันทึกผลด้วยมือไหม</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>การบันทึกผลการจ่ายและการแจ้งผู้ขาย</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>บันทึกด้วยมือต่อรายการจนกว่าได้สเปกไฟล์ผล</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>OQ-135 FR-PAY-103 P0-03</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>ตัวอย่างไฟล์ผลการโอนจากธนาคาร</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Q-83</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>การเงิน ตรวจสอบภายใน</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>ถ้ายกเลิกรอบจ่ายหรือสร้างไฟล์ใหม่หลังดาวน์โหลดไฟล์ไปแล้ว หรือบันทึกผลการจ่ายผิด ให้ระบบทำอย่างไร</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>กันการจ่ายซ้ำและ 50 ทวิ ที่ออกผิด</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>ยืนยันว่ายังไม่ได้ส่งธนาคารพร้อมเหตุผล · ใบที่ออกจากรอบติดธงในรอบถัดไป · ย้อนผลที่บันทึกแล้วได้ก่อนยื่น ภ.ง.ด. (ทำตอน go-live)</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>OQ-136 FR-PAY-101 FR-PAY-103</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Q-84</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>CFO</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>บัญชีธนาคารของบริษัทที่ใช้จ่ายผู้ขาย (และแม่แบบไฟล์ของธนาคาร) ใครเพิ่ม เปลี่ยน และอนุมัติ</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>บัญชีต้นทางของไฟล์จ่ายเงิน</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>การเงินเสนอ CFO อนุมัติแบบเดียวกับบัญชีผู้ขาย พร้อม step-up</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>OQ-137 FR-PAY-102</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Q-85</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>CEO ตรวจสอบภายใน</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>ให้ผู้ดูแล DOA ของบริษัทใช้ AI ร่างกฎ DOA จากระเบียบไหม (คนตรวจทุกข้อและอนุมัติแบบ 4 ตาเหมือนเดิม)</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>ความเป็นเจ้าของนโยบายอำนาจ (NG-12)</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>ใช้ได้เฉพาะคนของบริษัทที่มีสิทธิ์ร่าง DOA · ทีม BCS ใช้ไม่ได้</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>OQ-146 FR-AI-308</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>ระเบียบอำนาจอนุมัติฉบับปัจจุบัน</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Q-86</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>จัดซื้อ บัญชี</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>ค่าที่ AI อ่านจากเอกสารแบบไหนต้องให้คนยืนยันทีละช่อง</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>ภาระงานตรวจกับความเสี่ยงที่ค่าผิดหลุด</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>เงิน จำนวน เลขผู้เสียภาษี สาขา ประเภทคำขอ และค่าที่ AI ไม่มั่นใจ ยืนยันทีละช่อง ที่เหลือยืนยันรวม</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>OQ-147 BR-AI-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Q-87</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>กฎหมาย DPO</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>ให้ AI ตอบคำถามคัดกรอง (ผู้ขายประมวลผลข้อมูลส่วนบุคคล เข้าระบบ เข้าพื้นที่) แทนผู้ขอไหม</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>การขอ DPA และผู้ตรวจคู่ขนาน</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>ไม่ให้ AI ตอบ ผู้ขอตอบเอง</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>OQ-148 BR-FORM-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Q-88</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>กฎหมาย DPO</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>ข้อความและรูปที่พนักงานส่งในแชท LINE เพื่อขอซื้อ ให้เก็บไว้นานเท่าไร</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>ข้อมูลส่วนบุคคลในแชท (PDPA)</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>ข้อความ 7 วัน รูปที่ไม่ได้ใช้ 7 วัน รูปที่แนบเข้าคำขอเก็บตามอายุเอกสาร</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>OQ-162 FR-LINE-301</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Q-89</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>ผู้บริหาร IT</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>ผู้ที่ใช้แอป BCS Go ให้แจ้งเตือนในแอปแทน LINE หรือส่งทั้งสองทาง</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>แจ้งซ้ำสองที่และโควตา LINE</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>แทน LINE เมื่อผู้ใช้เปิดในแอป ส่งไม่ได้ย้อนไป LINE แล้วอีเมล</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>OQ-165 FR-PLT-301</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Q-90</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>CFO ตรวจสอบภายใน</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>ยืนยันด้วยลายนิ้วมือหรือใบหน้าในแอปใช้แทน PIN ได้ไหม และใช้เข้าระบบแทนรหัสผ่านได้ไหม</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>การยืนยันก่อนอนุมัติยอดสูงและการเข้าระบบ</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>แทน PIN ได้ทุกที่ที่ต้องยืนยัน ยังไม่ใช้แทนการเข้าระบบ</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>OQ-168 FR-AUTH-005</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Q-91</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>IT DPO</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>ข้อมูลตรวจรับที่บันทึกตอนไม่มีสัญญาณ เก็บในมือถือได้นานเท่าไร และต้องเข้ารหัสเพิ่มไหม</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>ข้อมูลในเครื่องที่หายหรือถูกขโมย</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>ไม่มีราคา ลบเมื่อส่งสำเร็จ ที่ยังไม่ส่งนานสุด 7 วัน ใช้การเข้ารหัสของเครื่อง</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>OQ-169 FR-PLT-301</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Q-92</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>บัญชี</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>ใบตรวจรับที่บันทึกตอนไม่มีสัญญาณ ให้ลงวันที่รับของจริงหรือวันที่ส่งเข้าระบบ</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>วันที่ในใบตรวจรับ รายงานสิ้นเดือน และวันคืนเงินประกัน</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>วันที่รับของจริงในเอกสาร ส่วนงบ รายงาน และกำหนดเวลานับเมื่อส่งเข้าระบบ</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>OQ-170 FR-PLT-301</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Q-93</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>หน้างาน จัดซื้อ</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>ให้ผู้ตรวจรับได้แจ้งเตือนทันทีเมื่อส่ง PO ให้ผู้ขายไหม</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>ผู้ตรวจรับรู้ก่อนของมาถึงหน้างาน</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>แจ้งทันทีทาง LINE หรือแอปพร้อมลิงก์หน้าตรวจรับ</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>OQ-171 NEW-64</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>B-01</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>BCS</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>ทีม BCS</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>LIFF ใช้ LINE MINI App หรือ LINE Login channel ใน production</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>การเผยแพร่และการ login ใน LINE</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>MINI App + ตรวจ ID token เอง</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>OQ-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>B-02</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>BCS</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>ทีม BCS</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>วิธีสร้าง PDF</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>คุณภาพภาษาไทยบนเอกสาร</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>ตัดสินแล้ว (ADR-044)</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>OQ-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>B-03</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>BCS</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>ทีม BCS</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>ยืนยันการประกาศพระราชกฤษฎีกาคง VAT 7%</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>อัตรา VAT ในระบบ</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>7% และให้ PLATFORM_ADMIN ยืนยัน</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>OQ-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>B-04</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>BCS</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>ทีม BCS</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>ปิดโมดูลขณะมีเอกสารค้าง</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>การเปลี่ยนแพ็กเกจ</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>ปฏิเสธและแสดงรายการเอกสาร</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>OQ-33</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>B-05</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>BCS</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>ทีม BCS</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>ผู้ให้บริการอีเมล hosting และที่เก็บไฟล์ของ production</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>ต้นทุนและที่ตั้งข้อมูล</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>ยังไม่ตัดสิน</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>ADR-031 ADR-032 ADR-033</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>B-06</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>BCS</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>ทีม BCS</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>ราคาและแพ็กเกจที่จะเสนอหลัง demo ระยะ 1</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>สัญญาและขอบเขต</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>ตามขนาดองค์กรและโมดูล</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>ADR-009</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
           <t>B-07</t>
         </is>
       </c>
-      <c r="B72" t="inlineStr">
+      <c r="B102" t="inlineStr">
         <is>
           <t>BCS</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr">
+      <c r="C102" t="inlineStr">
         <is>
           <t>ทีม BCS</t>
         </is>
       </c>
-      <c r="D72" t="inlineStr">
+      <c r="D102" t="inlineStr">
         <is>
           <t>บริการตรวจผู้ขายของสรรพากรและ DBD ยังเปิด และเรียกจาก hosting ได้หรือไม่</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr">
+      <c r="E102" t="inlineStr">
         <is>
           <t>การเติมข้อมูลผู้ขายอัตโนมัติ</t>
         </is>
       </c>
-      <c r="F72" t="inlineStr">
+      <c r="F102" t="inlineStr">
         <is>
           <t>โหมด stub จนกว่าจะทดสอบผ่าน</t>
         </is>
       </c>
-      <c r="G72" t="inlineStr">
+      <c r="G102" t="inlineStr">
         <is>
           <t>OQ-37</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>B-08</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>BCS</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>ทีม BCS</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>เกณฑ์ผ่านชุดประเมิน AI ชั้น demo กับเอกสารสังเคราะห์</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>เปิด AI ใน demo ระยะ 1</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>ฟิลด์สำคัญถูก ≥ 98% และค่าผิดทุกค่าถูกไฮไลต์ · ฟิลด์อื่น ≥ 90%</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>OQ-141 §12.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>B-09</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>BCS</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>ทีม BCS</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>ใช้ Claude API key ของ BCS ใน demo และ production อย่างไร และให้ credits AI ต่อองค์กรเดือนละเท่าไร</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>ค่าใช้จ่าย AI และการเปิด AI บน staging</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>key dev กับ key production แยกกันและมีวงเงิน · 20,000 credits ต่อเดือน (1 credit = 0.001 USD)</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>OQ-143 P0-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>B-10</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>BCS</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>ทีม BCS</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>ใช้ Claude รุ่นไหนกับ AI แต่ละงาน</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>ความแม่นและค่าใช้จ่าย</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>อ่านเอกสารและถามข้อมูล Sonnet 5.5 · เติมฟอร์มและสรุป Haiku 5.5 · ร่าง DOA Opus 5.5 · เปลี่ยนเมื่อผลประเมินชี้</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>OQ-145 BR-AI-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>B-11</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>BCS</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>ทีม BCS</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>ส่งการแจ้งเตือนในแอปผ่านบริการไหน และใช้ Firebase project ของใครใน demo</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>ต้นทุน ที่ตั้งข้อมูล และรายการ sub-processor</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>Firebase Cloud Messaging HTTP v1 ไม่เพิ่ม dependency · demo ใช้ project ของ BCS</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>OQ-164</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>B-12</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>BCS</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>ทีม BCS</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>แอป BCS Go เผยแพร่ใต้บัญชี store ของ BCS เป็นแอปเดียวทุกลูกค้าไหม</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>ค่าใช้จ่ายและการดูแลรุ่นของแอป</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>แอปเดียวใต้บัญชีของ BCS · demo ใช้ Android ติดตั้งเองและ PWA</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>OQ-166</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>B-13</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>BCS</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>ทีม BCS</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>ยืนยัน dependency ด้าน auth สำหรับยืนยันด้วยลายนิ้วมือในแอป: @simplewebauthn/server (แนะนำ) หรือ @better-auth/passkey</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>dependency ด้าน auth ต้องยืนยันก่อนติดตั้ง (§17.4) และปลั๊กอินเปิด endpoint ที่ต้องกั้นเพิ่ม</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>ยังไม่ติดตั้ง ใช้ PIN จนกว่าจะยืนยัน</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>OQ-167</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(sub-specs): P1-05 independent review of S6 S8 S9 S13 S17 and the shared base, decisions report
Six fresh-context reviewers recomputed every golden number (all match) and
checked each sub-spec against spec §1.6 §2 §4.11 §7 §8.11 §8.12 and the code.
Correctness fixes: chat approval of payment runs, stale bank-file downloads,
double use of received quantity across invoices, PO change approved below
progress, AI brief and AI log scope leaks, email-link step-up for new
subjects, reviewer-task step-up hooks, APP channel for policy decisions,
offline GR write lines. New OQ-138 (pay before due date) with its question.
docs/reports/p1-decisions.md lists all 88 decisions for P1-06 in plain Thai.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/inputs/BCS_inputs_p1.xlsx
+++ b/docs/inputs/BCS_inputs_p1.xlsx
@@ -70354,7 +70354,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I108"/>
+  <dimension ref="A1:I109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -73703,37 +73703,32 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>CEO ตรวจสอบภายใน</t>
+          <t>การเงิน CFO</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>ให้ผู้ดูแล DOA ของบริษัทใช้ AI ร่างกฎ DOA จากระเบียบไหม (คนตรวจทุกข้อและอนุมัติแบบ 4 ตาเหมือนเดิม)</t>
+          <t>จ่ายใบแจ้งหนี้ที่ยังไม่ถึงวันครบกำหนดในรอบจ่ายได้ไหม และต้องใส่เหตุผลหรือไม่</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>ความเป็นเจ้าของนโยบายอำนาจ (NG-12)</t>
+          <t>จ่ายก่อนกำหนดทำให้เงินออกเร็วกว่าที่จำเป็น</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>ใช้ได้เฉพาะคนของบริษัทที่มีสิทธิ์ร่าง DOA · ทีม BCS ใช้ไม่ได้</t>
+          <t>ได้ ใบมีป้าย "จ่ายก่อนกำหนด" ที่ผู้อนุมัติเห็น ไม่บังคับเหตุผล</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>OQ-146 FR-AI-308</t>
-        </is>
-      </c>
-      <c r="I87" t="inlineStr">
-        <is>
-          <t>ระเบียบอำนาจอนุมัติฉบับปัจจุบัน</t>
+          <t>OQ-138 FR-PAY-101</t>
         </is>
       </c>
     </row>
@@ -73745,32 +73740,37 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>จัดซื้อ บัญชี</t>
+          <t>CEO ตรวจสอบภายใน</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>ค่าที่ AI อ่านจากเอกสารแบบไหนต้องให้คนยืนยันทีละช่อง</t>
+          <t>ให้ผู้ดูแล DOA ของบริษัทใช้ AI ร่างกฎ DOA จากระเบียบไหม (คนตรวจทุกข้อและอนุมัติแบบ 4 ตาเหมือนเดิม)</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>ภาระงานตรวจกับความเสี่ยงที่ค่าผิดหลุด</t>
+          <t>ความเป็นเจ้าของนโยบายอำนาจ (NG-12)</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>เงิน จำนวน เลขผู้เสียภาษี สาขา ประเภทคำขอ และค่าที่ AI ไม่มั่นใจ ยืนยันทีละช่อง ที่เหลือยืนยันรวม</t>
+          <t>ใช้ได้เฉพาะคนของบริษัทที่มีสิทธิ์ร่าง DOA · ทีม BCS ใช้ไม่ได้</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>OQ-147 BR-AI-02</t>
+          <t>OQ-146 FR-AI-308</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>ระเบียบอำนาจอนุมัติฉบับปัจจุบัน</t>
         </is>
       </c>
     </row>
@@ -73782,32 +73782,32 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>กฎหมาย DPO</t>
+          <t>จัดซื้อ บัญชี</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>ให้ AI ตอบคำถามคัดกรอง (ผู้ขายประมวลผลข้อมูลส่วนบุคคล เข้าระบบ เข้าพื้นที่) แทนผู้ขอไหม</t>
+          <t>ค่าที่ AI อ่านจากเอกสารแบบไหนต้องให้คนยืนยันทีละช่อง</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>การขอ DPA และผู้ตรวจคู่ขนาน</t>
+          <t>ภาระงานตรวจกับความเสี่ยงที่ค่าผิดหลุด</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>ไม่ให้ AI ตอบ ผู้ขอตอบเอง</t>
+          <t>เงิน จำนวน เลขผู้เสียภาษี สาขา ประเภทคำขอ และค่าที่ AI ไม่มั่นใจ ยืนยันทีละช่อง ที่เหลือยืนยันรวม</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>OQ-148 BR-FORM-05</t>
+          <t>OQ-147 BR-AI-02</t>
         </is>
       </c>
     </row>
@@ -73829,22 +73829,22 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>ข้อความและรูปที่พนักงานส่งในแชท LINE เพื่อขอซื้อ ให้เก็บไว้นานเท่าไร</t>
+          <t>ให้ AI ตอบคำถามคัดกรอง (ผู้ขายประมวลผลข้อมูลส่วนบุคคล เข้าระบบ เข้าพื้นที่) แทนผู้ขอไหม</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>ข้อมูลส่วนบุคคลในแชท (PDPA)</t>
+          <t>การขอ DPA และผู้ตรวจคู่ขนาน</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>ข้อความ 7 วัน รูปที่ไม่ได้ใช้ 7 วัน รูปที่แนบเข้าคำขอเก็บตามอายุเอกสาร</t>
+          <t>ไม่ให้ AI ตอบ ผู้ขอตอบเอง</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>OQ-162 FR-LINE-301</t>
+          <t>OQ-148 BR-FORM-05</t>
         </is>
       </c>
     </row>
@@ -73861,27 +73861,27 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>ผู้บริหาร IT</t>
+          <t>กฎหมาย DPO</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>ผู้ที่ใช้แอป BCS Go ให้แจ้งเตือนในแอปแทน LINE หรือส่งทั้งสองทาง</t>
+          <t>ข้อความและรูปที่พนักงานส่งในแชท LINE เพื่อขอซื้อ ให้เก็บไว้นานเท่าไร</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>แจ้งซ้ำสองที่และโควตา LINE</t>
+          <t>ข้อมูลส่วนบุคคลในแชท (PDPA)</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>แทน LINE เมื่อผู้ใช้เปิดในแอป ส่งไม่ได้ย้อนไป LINE แล้วอีเมล</t>
+          <t>ข้อความ 7 วัน รูปที่ไม่ได้ใช้ 7 วัน รูปที่แนบเข้าคำขอเก็บตามอายุเอกสาร</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>OQ-165 FR-PLT-301</t>
+          <t>OQ-162 FR-LINE-301</t>
         </is>
       </c>
     </row>
@@ -73893,32 +73893,32 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>CFO ตรวจสอบภายใน</t>
+          <t>ผู้บริหาร IT</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>ยืนยันด้วยลายนิ้วมือหรือใบหน้าในแอปใช้แทน PIN ได้ไหม และใช้เข้าระบบแทนรหัสผ่านได้ไหม</t>
+          <t>ผู้ที่ใช้แอป BCS Go ให้แจ้งเตือนในแอปแทน LINE หรือส่งทั้งสองทาง</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>การยืนยันก่อนอนุมัติยอดสูงและการเข้าระบบ</t>
+          <t>แจ้งซ้ำสองที่และโควตา LINE</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>แทน PIN ได้ทุกที่ที่ต้องยืนยัน ยังไม่ใช้แทนการเข้าระบบ</t>
+          <t>แทน LINE เมื่อผู้ใช้เปิดในแอป ส่งไม่ได้ย้อนไป LINE แล้วอีเมล</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>OQ-168 FR-AUTH-005</t>
+          <t>OQ-165 FR-PLT-301</t>
         </is>
       </c>
     </row>
@@ -73930,32 +73930,32 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>IT DPO</t>
+          <t>CFO ตรวจสอบภายใน</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>ข้อมูลตรวจรับที่บันทึกตอนไม่มีสัญญาณ เก็บในมือถือได้นานเท่าไร และต้องเข้ารหัสเพิ่มไหม</t>
+          <t>ยืนยันด้วยลายนิ้วมือหรือใบหน้าในแอปใช้แทน PIN ได้ไหม และใช้เข้าระบบแทนรหัสผ่านได้ไหม</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>ข้อมูลในเครื่องที่หายหรือถูกขโมย</t>
+          <t>การยืนยันก่อนอนุมัติยอดสูงและการเข้าระบบ</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>ไม่มีราคา ลบเมื่อส่งสำเร็จ ที่ยังไม่ส่งนานสุด 7 วัน ใช้การเข้ารหัสของเครื่อง</t>
+          <t>แทน PIN ได้ทุกที่ที่ต้องยืนยัน ยังไม่ใช้แทนการเข้าระบบ</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>OQ-169 FR-PLT-301</t>
+          <t>OQ-168 FR-AUTH-005</t>
         </is>
       </c>
     </row>
@@ -73967,32 +73967,32 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>บัญชี</t>
+          <t>IT DPO</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>ใบตรวจรับที่บันทึกตอนไม่มีสัญญาณ ให้ลงวันที่รับของจริงหรือวันที่ส่งเข้าระบบ</t>
+          <t>ข้อมูลตรวจรับที่บันทึกตอนไม่มีสัญญาณ เก็บในมือถือได้นานเท่าไร และต้องเข้ารหัสเพิ่มไหม</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>วันที่ในใบตรวจรับ รายงานสิ้นเดือน และวันคืนเงินประกัน</t>
+          <t>ข้อมูลในเครื่องที่หายหรือถูกขโมย</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>วันที่รับของจริงในเอกสาร ส่วนงบ รายงาน และกำหนดเวลานับเมื่อส่งเข้าระบบ</t>
+          <t>ไม่มีราคา ลบเมื่อส่งสำเร็จ ที่ยังไม่ส่งนานสุด 7 วัน ใช้การเข้ารหัสของเครื่อง</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>OQ-170 FR-PLT-301</t>
+          <t>OQ-169 FR-PLT-301</t>
         </is>
       </c>
     </row>
@@ -74004,76 +74004,76 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>หน้างาน จัดซื้อ</t>
+          <t>บัญชี</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>ให้ผู้ตรวจรับได้แจ้งเตือนทันทีเมื่อส่ง PO ให้ผู้ขายไหม</t>
+          <t>ใบตรวจรับที่บันทึกตอนไม่มีสัญญาณ ให้ลงวันที่รับของจริงหรือวันที่ส่งเข้าระบบ</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>ผู้ตรวจรับรู้ก่อนของมาถึงหน้างาน</t>
+          <t>วันที่ในใบตรวจรับ รายงานสิ้นเดือน และวันคืนเงินประกัน</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>แจ้งทันทีทาง LINE หรือแอปพร้อมลิงก์หน้าตรวจรับ</t>
+          <t>วันที่รับของจริงในเอกสาร ส่วนงบ รายงาน และกำหนดเวลานับเมื่อส่งเข้าระบบ</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>OQ-171 NEW-64</t>
+          <t>OQ-170 FR-PLT-301</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>B-01</t>
+          <t>Q-94</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>BCS</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>ทีม BCS</t>
+          <t>หน้างาน จัดซื้อ</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>LIFF ใช้ LINE MINI App หรือ LINE Login channel ใน production</t>
+          <t>ให้ผู้ตรวจรับได้แจ้งเตือนทันทีเมื่อส่ง PO ให้ผู้ขายไหม</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>การเผยแพร่และการ login ใน LINE</t>
+          <t>ผู้ตรวจรับรู้ก่อนของมาถึงหน้างาน</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>MINI App + ตรวจ ID token เอง</t>
+          <t>แจ้งทันทีทาง LINE หรือแอปพร้อมลิงก์หน้าตรวจรับ</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>OQ-16</t>
+          <t>OQ-171 NEW-64</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>B-02</t>
+          <t>B-01</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -74088,29 +74088,29 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>วิธีสร้าง PDF</t>
+          <t>LIFF ใช้ LINE MINI App หรือ LINE Login channel ใน production</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>คุณภาพภาษาไทยบนเอกสาร</t>
+          <t>การเผยแพร่และการ login ใน LINE</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>ตัดสินแล้ว (ADR-044)</t>
+          <t>MINI App + ตรวจ ID token เอง</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>OQ-18</t>
+          <t>OQ-16</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>B-03</t>
+          <t>B-02</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -74125,29 +74125,29 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>ยืนยันการประกาศพระราชกฤษฎีกาคง VAT 7%</t>
+          <t>วิธีสร้าง PDF</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>อัตรา VAT ในระบบ</t>
+          <t>คุณภาพภาษาไทยบนเอกสาร</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>7% และให้ PLATFORM_ADMIN ยืนยัน</t>
+          <t>ตัดสินแล้ว (ADR-044)</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>OQ-29</t>
+          <t>OQ-18</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>B-04</t>
+          <t>B-03</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -74162,29 +74162,29 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>ปิดโมดูลขณะมีเอกสารค้าง</t>
+          <t>ยืนยันการประกาศพระราชกฤษฎีกาคง VAT 7%</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>การเปลี่ยนแพ็กเกจ</t>
+          <t>อัตรา VAT ในระบบ</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>ปฏิเสธและแสดงรายการเอกสาร</t>
+          <t>7% และให้ PLATFORM_ADMIN ยืนยัน</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>OQ-33</t>
+          <t>OQ-29</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>B-05</t>
+          <t>B-04</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -74199,29 +74199,29 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>ผู้ให้บริการอีเมล hosting และที่เก็บไฟล์ของ production</t>
+          <t>ปิดโมดูลขณะมีเอกสารค้าง</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>ต้นทุนและที่ตั้งข้อมูล</t>
+          <t>การเปลี่ยนแพ็กเกจ</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>ยังไม่ตัดสิน</t>
+          <t>ปฏิเสธและแสดงรายการเอกสาร</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>ADR-031 ADR-032 ADR-033</t>
+          <t>OQ-33</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>B-06</t>
+          <t>B-05</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -74236,29 +74236,29 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>ราคาและแพ็กเกจที่จะเสนอหลัง demo ระยะ 1</t>
+          <t>ผู้ให้บริการอีเมล hosting และที่เก็บไฟล์ของ production</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>สัญญาและขอบเขต</t>
+          <t>ต้นทุนและที่ตั้งข้อมูล</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>ตามขนาดองค์กรและโมดูล</t>
+          <t>ยังไม่ตัดสิน</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>ADR-009</t>
+          <t>ADR-031 ADR-032 ADR-033</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>B-07</t>
+          <t>B-06</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -74273,29 +74273,29 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>บริการตรวจผู้ขายของสรรพากรและ DBD ยังเปิด และเรียกจาก hosting ได้หรือไม่</t>
+          <t>ราคาและแพ็กเกจที่จะเสนอหลัง demo ระยะ 1</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>การเติมข้อมูลผู้ขายอัตโนมัติ</t>
+          <t>สัญญาและขอบเขต</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>โหมด stub จนกว่าจะทดสอบผ่าน</t>
+          <t>ตามขนาดองค์กรและโมดูล</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>OQ-37</t>
+          <t>ADR-009</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>B-08</t>
+          <t>B-07</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -74310,29 +74310,29 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>เกณฑ์ผ่านชุดประเมิน AI ชั้น demo กับเอกสารสังเคราะห์</t>
+          <t>บริการตรวจผู้ขายของสรรพากรและ DBD ยังเปิด และเรียกจาก hosting ได้หรือไม่</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>เปิด AI ใน demo ระยะ 1</t>
+          <t>การเติมข้อมูลผู้ขายอัตโนมัติ</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>ฟิลด์สำคัญถูก ≥ 98% และค่าผิดทุกค่าถูกไฮไลต์ · ฟิลด์อื่น ≥ 90%</t>
+          <t>โหมด stub จนกว่าจะทดสอบผ่าน</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>OQ-141 §12.4</t>
+          <t>OQ-37</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>B-09</t>
+          <t>B-08</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -74347,29 +74347,29 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>ใช้ Claude API key ของ BCS ใน demo และ production อย่างไร และให้ credits AI ต่อองค์กรเดือนละเท่าไร</t>
+          <t>เกณฑ์ผ่านชุดประเมิน AI ชั้น demo กับเอกสารสังเคราะห์</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>ค่าใช้จ่าย AI และการเปิด AI บน staging</t>
+          <t>เปิด AI ใน demo ระยะ 1</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>key dev กับ key production แยกกันและมีวงเงิน · 20,000 credits ต่อเดือน (1 credit = 0.001 USD)</t>
+          <t>ฟิลด์สำคัญถูก ≥ 98% และค่าผิดทุกค่าถูกไฮไลต์ · ฟิลด์อื่น ≥ 90%</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>OQ-143 P0-13</t>
+          <t>OQ-141 §12.4</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>B-10</t>
+          <t>B-09</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -74384,29 +74384,29 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>ใช้ Claude รุ่นไหนกับ AI แต่ละงาน</t>
+          <t>ใช้ Claude API key ของ BCS ใน demo และ production อย่างไร และให้ credits AI ต่อองค์กรเดือนละเท่าไร</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>ความแม่นและค่าใช้จ่าย</t>
+          <t>ค่าใช้จ่าย AI และการเปิด AI บน staging</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>อ่านเอกสารและถามข้อมูล Sonnet 5.5 · เติมฟอร์มและสรุป Haiku 5.5 · ร่าง DOA Opus 5.5 · เปลี่ยนเมื่อผลประเมินชี้</t>
+          <t>key dev กับ key production แยกกันและมีวงเงิน · 20,000 credits ต่อเดือน (1 credit = 0.001 USD)</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>OQ-145 BR-AI-09</t>
+          <t>OQ-143 P0-13</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>B-11</t>
+          <t>B-10</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -74421,29 +74421,29 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>ส่งการแจ้งเตือนในแอปผ่านบริการไหน และใช้ Firebase project ของใครใน demo</t>
+          <t>ใช้ Claude รุ่นไหนกับ AI แต่ละงาน</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>ต้นทุน ที่ตั้งข้อมูล และรายการ sub-processor</t>
+          <t>ความแม่นและค่าใช้จ่าย</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>Firebase Cloud Messaging HTTP v1 ไม่เพิ่ม dependency · demo ใช้ project ของ BCS</t>
+          <t>อ่านเอกสารและถามข้อมูล Sonnet 5.5 · เติมฟอร์มและสรุป Haiku 5.5 · ร่าง DOA Opus 5.5 · เปลี่ยนเมื่อผลประเมินชี้</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>OQ-164</t>
+          <t>OQ-145 BR-AI-09</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>B-12</t>
+          <t>B-11</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -74458,57 +74458,94 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>แอป BCS Go เผยแพร่ใต้บัญชี store ของ BCS เป็นแอปเดียวทุกลูกค้าไหม</t>
+          <t>ส่งการแจ้งเตือนในแอปผ่านบริการไหน และใช้ Firebase project ของใครใน demo</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>ค่าใช้จ่ายและการดูแลรุ่นของแอป</t>
+          <t>ต้นทุน ที่ตั้งข้อมูล และรายการ sub-processor</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>แอปเดียวใต้บัญชีของ BCS · demo ใช้ Android ติดตั้งเองและ PWA</t>
+          <t>Firebase Cloud Messaging HTTP v1 ไม่เพิ่ม dependency · demo ใช้ project ของ BCS</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>OQ-166</t>
+          <t>OQ-164</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
+          <t>B-12</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>BCS</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>ทีม BCS</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>แอป BCS Go เผยแพร่ใต้บัญชี store ของ BCS เป็นแอปเดียวทุกลูกค้าไหม</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>ค่าใช้จ่ายและการดูแลรุ่นของแอป</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>แอปเดียวใต้บัญชีของ BCS · demo ใช้ Android ติดตั้งเองและ PWA</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>OQ-166</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
           <t>B-13</t>
         </is>
       </c>
-      <c r="B108" t="inlineStr">
+      <c r="B109" t="inlineStr">
         <is>
           <t>BCS</t>
         </is>
       </c>
-      <c r="C108" t="inlineStr">
+      <c r="C109" t="inlineStr">
         <is>
           <t>ทีม BCS</t>
         </is>
       </c>
-      <c r="D108" t="inlineStr">
+      <c r="D109" t="inlineStr">
         <is>
           <t>ยืนยัน dependency ด้าน auth สำหรับยืนยันด้วยลายนิ้วมือในแอป: @simplewebauthn/server (แนะนำ) หรือ @better-auth/passkey</t>
         </is>
       </c>
-      <c r="E108" t="inlineStr">
+      <c r="E109" t="inlineStr">
         <is>
           <t>dependency ด้าน auth ต้องยืนยันก่อนติดตั้ง (§17.4) และปลั๊กอินเปิด endpoint ที่ต้องกั้นเพิ่ม</t>
         </is>
       </c>
-      <c r="F108" t="inlineStr">
+      <c r="F109" t="inlineStr">
         <is>
           <t>ยังไม่ติดตั้ง ใช้ PIN จนกว่าจะยืนยัน</t>
         </is>
       </c>
-      <c r="G108" t="inlineStr">
+      <c r="G109" t="inlineStr">
         <is>
           <t>OQ-167</t>
         </is>

</xml_diff>

<commit_message>
feat(seed): P1-07 part 6 phase-1 data: DOA-SIMEC version 1 with the new types, PAY AI BCS_GO on
- scripts/inputs_p1: the 14 draft rules of the six new document types join sheet DOA version 1 (OQ-40 draft);
  sheet DOA_P1_Draft removed; validate_inputs.py knows 11 types, no band on BANK_ACCOUNT_CHANGE, PAY's types
  required in the p1 file; p1_texts.py README and Inputs rows; workbook regenerated with make.py
- seed of the p1 workbook switches PAY AI BCS_GO on once after the DOA (contractRef SEED-P1, module_enabled
  events, refused when the DOA lacks a module's rules); the demo keeps CORE alone; the DOA sheet takes every type
- pnpm db:reset:p1: DOA-SIMEC version 1 with 22 rules, 3 modules switched on (125 s)
- tests: FR-PLT-007 AC4 AC5

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/inputs/BCS_inputs_p1.xlsx
+++ b/docs/inputs/BCS_inputs_p1.xlsx
@@ -16,24 +16,23 @@
     <sheet name="Users" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="DOA" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="DOA_Policy" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="DOA_P1_Draft" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Workflow_Reviewers" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Budget" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="CostCenters" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="GL_Accounts" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Suppliers" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="SupplierPayment" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="Banks" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="Items" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="Sites" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="RequestTypes" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="Holidays" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="Settings" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="WHT_Types" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="CompanyBankAccounts" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="Request_History" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="DocSamples" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet name="Scenarios" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="Workflow_Reviewers" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Budget" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="CostCenters" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="GL_Accounts" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Suppliers" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="SupplierPayment" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Banks" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Items" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Sites" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="RequestTypes" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="Holidays" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="Settings" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="WHT_Types" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="CompanyBankAccounts" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="Request_History" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="DocSamples" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="Scenarios" sheetId="26" state="visible" r:id="rId26"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -692,12 +691,12 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>DOA_P1_Draft · Workflow_Reviewers</t>
+          <t>Workflow_Reviewers</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>ร่างวงเงินของเอกสารชนิดใหม่และผู้ตรวจคู่ขนานของระยะ 1 · seed ยังไม่อ่าน · sub-spec ของ S6 S8 S9 ตัดสินร่วมกับผู้ใช้</t>
+          <t>ร่างผู้ตรวจคู่ขนานของระยะ 1 · seed ยังไม่อ่าน · S6 อ่านเอง</t>
         </is>
       </c>
     </row>
@@ -803,678 +802,6 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:I16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="27" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="60" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="6" t="inlineStr">
-        <is>
-          <t>documentType</t>
-        </is>
-      </c>
-      <c r="B1" s="6" t="inlineStr">
-        <is>
-          <t>ruleCode</t>
-        </is>
-      </c>
-      <c r="C1" s="6" t="inlineStr">
-        <is>
-          <t>gt</t>
-        </is>
-      </c>
-      <c r="D1" s="6" t="inlineStr">
-        <is>
-          <t>lte</t>
-        </is>
-      </c>
-      <c r="E1" s="6" t="inlineStr">
-        <is>
-          <t>approverKind</t>
-        </is>
-      </c>
-      <c r="F1" s="6" t="inlineStr">
-        <is>
-          <t>approverPosition</t>
-        </is>
-      </c>
-      <c r="G1" s="6" t="inlineStr">
-        <is>
-          <t>slaBusinessHours</t>
-        </is>
-      </c>
-      <c r="H1" s="6" t="inlineStr">
-        <is>
-          <t>descriptionTh</t>
-        </is>
-      </c>
-      <c r="I1" s="6" t="inlineStr">
-        <is>
-          <t>ref</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="5" t="inlineStr">
-        <is>
-          <t>ประเภทเอกสารใหม่ของระยะ 1</t>
-        </is>
-      </c>
-      <c r="B2" s="5" t="inlineStr">
-        <is>
-          <t>รหัสข้อ</t>
-        </is>
-      </c>
-      <c r="C2" s="5" t="inlineStr">
-        <is>
-          <t>มากกว่า (บาท)</t>
-        </is>
-      </c>
-      <c r="D2" s="5" t="inlineStr">
-        <is>
-          <t>ไม่เกิน (บาท)</t>
-        </is>
-      </c>
-      <c r="E2" s="5" t="inlineStr">
-        <is>
-          <t>วิธีหาผู้อนุมัติ</t>
-        </is>
-      </c>
-      <c r="F2" s="5" t="inlineStr">
-        <is>
-          <t>ตำแหน่ง</t>
-        </is>
-      </c>
-      <c r="G2" s="5" t="inlineStr">
-        <is>
-          <t>SLA ชั่วโมงทำการ</t>
-        </is>
-      </c>
-      <c r="H2" s="5" t="inlineStr">
-        <is>
-          <t>คำอธิบาย (ร่าง รอลูกค้ายืนยัน · seed ยังไม่อ่าน)</t>
-        </is>
-      </c>
-      <c r="I2" s="5" t="inlineStr">
-        <is>
-          <t>FR</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>BUDGET_TRANSFER</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>BT-01</t>
-        </is>
-      </c>
-      <c r="C3" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D3" s="7" t="n">
-        <v>100000</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>POSITION_OF_DEPARTMENT</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>DM</t>
-        </is>
-      </c>
-      <c r="G3" t="n">
-        <v>8</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>โอนงบระหว่างบรรทัดไม่เกิน 100,000 → ผู้จัดการฝ่ายเจ้าของงบต้นทาง</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>FR-BUD-103</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>BUDGET_TRANSFER</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>BT-02</t>
-        </is>
-      </c>
-      <c r="C4" s="7" t="n">
-        <v>100000</v>
-      </c>
-      <c r="D4" s="7" t="n">
-        <v>500000</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>POSITION_OF_DEPARTMENT</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>VP</t>
-        </is>
-      </c>
-      <c r="G4" t="n">
-        <v>8</v>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>โอนงบเกิน 100,000 ถึง 500,000 → รองกรรมการผู้จัดการสายงาน</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>FR-BUD-103</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>BUDGET_TRANSFER</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>BT-03</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="n">
-        <v>500000</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>POSITION_OF_ORG</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>CFO</t>
-        </is>
-      </c>
-      <c r="G5" t="n">
-        <v>16</v>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>โอนงบเกิน 500,000 → CFO</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>FR-BUD-103</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>OVER_BUDGET</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>OB-01</t>
-        </is>
-      </c>
-      <c r="C6" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D6" s="7" t="n">
-        <v>50000</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>POSITION_OF_DEPARTMENT</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>VP</t>
-        </is>
-      </c>
-      <c r="G6" t="n">
-        <v>8</v>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>อนุมัติเกินงบไม่เกิน 50,000 → รองกรรมการผู้จัดการสายงาน</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>FR-BUD-101</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>OVER_BUDGET</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>OB-02</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D7" s="7" t="n">
-        <v>500000</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>POSITION_OF_ORG</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>CFO</t>
-        </is>
-      </c>
-      <c r="G7" t="n">
-        <v>16</v>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>อนุมัติเกินงบเกิน 50,000 ถึง 500,000 → CFO</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>FR-BUD-101</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>OVER_BUDGET</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>OB-03</t>
-        </is>
-      </c>
-      <c r="C8" s="7" t="n">
-        <v>500000</v>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>POSITION_OF_ORG</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>CEO</t>
-        </is>
-      </c>
-      <c r="G8" t="n">
-        <v>16</v>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>อนุมัติเกินงบเกิน 500,000 → กรรมการผู้จัดการ</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>FR-BUD-101</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>INVOICE_EXCEPTION</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>IE-01</t>
-        </is>
-      </c>
-      <c r="C9" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" s="7" t="n">
-        <v>20000</v>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>POSITION_OF_DEPARTMENT</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>DM</t>
-        </is>
-      </c>
-      <c r="G9" t="n">
-        <v>8</v>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>ใบแจ้งหนี้ต่างจาก PO นอกเกณฑ์ ส่วนต่างไม่เกิน 20,000 → ผู้จัดการฝ่ายเจ้าของงบ</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>FR-AP-103</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>INVOICE_EXCEPTION</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>IE-02</t>
-        </is>
-      </c>
-      <c r="C10" s="7" t="n">
-        <v>20000</v>
-      </c>
-      <c r="D10" s="7" t="n">
-        <v>200000</v>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>POSITION_OF_DEPARTMENT</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>VP</t>
-        </is>
-      </c>
-      <c r="G10" t="n">
-        <v>8</v>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>ส่วนต่างเกิน 20,000 ถึง 200,000 → รองกรรมการผู้จัดการสายงาน</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>FR-AP-103</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>INVOICE_EXCEPTION</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>IE-03</t>
-        </is>
-      </c>
-      <c r="C11" s="7" t="n">
-        <v>200000</v>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>POSITION_OF_ORG</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>CFO</t>
-        </is>
-      </c>
-      <c r="G11" t="n">
-        <v>16</v>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>ส่วนต่างเกิน 200,000 → CFO</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>FR-AP-103</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>PO_CHANGE</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>PC-01</t>
-        </is>
-      </c>
-      <c r="C12" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D12" s="7" t="n">
-        <v>1000000</v>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>POSITION_OF_ORG</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>COO</t>
-        </is>
-      </c>
-      <c r="G12" t="n">
-        <v>8</v>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>แก้ PO ที่ยอดใหม่ไม่เกิน 1,000,000 → COO</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>FR-AP-107</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>PO_CHANGE</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>PC-02</t>
-        </is>
-      </c>
-      <c r="C13" s="7" t="n">
-        <v>1000000</v>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>POSITION_OF_ORG</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>CEO</t>
-        </is>
-      </c>
-      <c r="G13" t="n">
-        <v>16</v>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>แก้ PO ที่ยอดใหม่เกิน 1,000,000 → กรรมการผู้จัดการ</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>FR-AP-107</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>PAYMENT_RUN</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>PAY-01</t>
-        </is>
-      </c>
-      <c r="C14" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D14" s="7" t="n">
-        <v>5000000</v>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>POSITION_OF_ORG</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>CFO</t>
-        </is>
-      </c>
-      <c r="G14" t="n">
-        <v>8</v>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>รอบจ่ายไม่เกิน 5,000,000 → CFO (ผู้เตรียมห้ามอนุมัติ BR-SOD-04)</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>FR-PAY-101</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>PAYMENT_RUN</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>PAY-02</t>
-        </is>
-      </c>
-      <c r="C15" s="7" t="n">
-        <v>5000000</v>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>POSITION_OF_ORG</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>CEO</t>
-        </is>
-      </c>
-      <c r="G15" t="n">
-        <v>16</v>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>รอบจ่ายเกิน 5,000,000 → กรรมการผู้จัดการ</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>FR-PAY-101</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>BANK_ACCOUNT_CHANGE</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>BA-01</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>POSITION_OF_ORG</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>CFO</t>
-        </is>
-      </c>
-      <c r="G16" t="n">
-        <v>8</v>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>เพิ่มหรือเปลี่ยนบัญชีรับเงินของผู้ขาย → CFO (ผู้แก้ห้ามอนุมัติ BR-SOD-05)</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>FR-PAY-102</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1908,7 +1235,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6137,7 +5464,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6632,7 +5959,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7067,7 +6394,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -16398,7 +15725,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -25844,7 +25171,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -26084,7 +25411,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -31413,7 +30740,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -31662,6 +30989,288 @@
       <c r="C14" t="inlineStr">
         <is>
           <t>คลังวัสดุกลาง บางพลี สมุทรปราการ (สมมติ)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="27" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>nameTh</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>documentType</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>descriptionTh</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>keyFields</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>attachmentRule</t>
+        </is>
+      </c>
+      <c r="G1" s="6" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>รหัส (ต้องมีฟอร์มใน prisma/seed/forms.yaml)</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>ชื่อบนการ์ด</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>ชนิดเอกสาร</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>ใช้เมื่อไร</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>ฟิลด์สำคัญ</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>กฎเอกสารแนบ</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>ใช้งาน (Y/N)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>BUY_GOODS</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ซื้อของ</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>PURCHASE_REQUEST</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>วัสดุก่อสร้าง อะไหล่ อุปกรณ์ความปลอดภัย และสินค้าทั่วไป</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>รายการ จำนวน หน่วย ราคาประมาณ สถานที่ส่ง วันที่ต้องใช้ บรรทัดงบ</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>ATT-QUOTES</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>HIRE_SERVICE</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>จ้างบริการ</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>PURCHASE_REQUEST</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>เช่าเครื่องจักร รปภ. ทำความสะอาด ทดสอบวัสดุ ที่ปรึกษา และอบรม</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>ขอบเขตงาน ระยะเวลา วันสิ้นสุดบริการ ราคาประมาณ ใบเสนอราคา บรรทัดงบ · คำถามคัดกรอง 3 ข้อ</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>ATT-QUOTES · ATT-DPA</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>CONTRACT_WORK</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>จ้างเหมา</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>PURCHASE_REQUEST</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>งานเหมาช่วงที่มีงวดงาน เช่น เสาเข็ม โครงสร้างเหล็ก งานระบบ งานถนน</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>ขอบเขตงาน งวดงาน ไซต์ ราคาประมาณ บรรทัดงบ</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>ATT-QUOTES</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>IT_PURCHASE</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ซื้ออุปกรณ์/ซอฟต์แวร์ไอที</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>PURCHASE_REQUEST</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>คอมพิวเตอร์ อุปกรณ์เครือข่าย ซอฟต์แวร์ และไลเซนส์</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>หมวด (HARDWARE/SOFTWARE) รายการ จำนวน ราคาประมาณ assetTag วันสิ้นสุดไลเซนส์ · คำถามคัดกรอง 3 ข้อ</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>ATT-QUOTES · ATT-DPA</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>NEW_SUPPLIER</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ขอเพิ่มผู้ขายรายใหม่</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>SUPPLIER_REQUEST</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>ผู้ขายที่ยังไม่อยู่ในทะเบียน</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>ชื่อ เลขผู้เสียภาษี สาขา อีเมล เหตุผล</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -33450,7 +33059,7 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>DOA_P1_Draft</t>
+          <t>DOA</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
@@ -33517,288 +33126,6 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="27" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="6" t="inlineStr">
-        <is>
-          <t>code</t>
-        </is>
-      </c>
-      <c r="B1" s="6" t="inlineStr">
-        <is>
-          <t>nameTh</t>
-        </is>
-      </c>
-      <c r="C1" s="6" t="inlineStr">
-        <is>
-          <t>documentType</t>
-        </is>
-      </c>
-      <c r="D1" s="6" t="inlineStr">
-        <is>
-          <t>descriptionTh</t>
-        </is>
-      </c>
-      <c r="E1" s="6" t="inlineStr">
-        <is>
-          <t>keyFields</t>
-        </is>
-      </c>
-      <c r="F1" s="6" t="inlineStr">
-        <is>
-          <t>attachmentRule</t>
-        </is>
-      </c>
-      <c r="G1" s="6" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="5" t="inlineStr">
-        <is>
-          <t>รหัส (ต้องมีฟอร์มใน prisma/seed/forms.yaml)</t>
-        </is>
-      </c>
-      <c r="B2" s="5" t="inlineStr">
-        <is>
-          <t>ชื่อบนการ์ด</t>
-        </is>
-      </c>
-      <c r="C2" s="5" t="inlineStr">
-        <is>
-          <t>ชนิดเอกสาร</t>
-        </is>
-      </c>
-      <c r="D2" s="5" t="inlineStr">
-        <is>
-          <t>ใช้เมื่อไร</t>
-        </is>
-      </c>
-      <c r="E2" s="5" t="inlineStr">
-        <is>
-          <t>ฟิลด์สำคัญ</t>
-        </is>
-      </c>
-      <c r="F2" s="5" t="inlineStr">
-        <is>
-          <t>กฎเอกสารแนบ</t>
-        </is>
-      </c>
-      <c r="G2" s="5" t="inlineStr">
-        <is>
-          <t>ใช้งาน (Y/N)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>BUY_GOODS</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>ซื้อของ</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>PURCHASE_REQUEST</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>วัสดุก่อสร้าง อะไหล่ อุปกรณ์ความปลอดภัย และสินค้าทั่วไป</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>รายการ จำนวน หน่วย ราคาประมาณ สถานที่ส่ง วันที่ต้องใช้ บรรทัดงบ</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>ATT-QUOTES</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>HIRE_SERVICE</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>จ้างบริการ</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>PURCHASE_REQUEST</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>เช่าเครื่องจักร รปภ. ทำความสะอาด ทดสอบวัสดุ ที่ปรึกษา และอบรม</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>ขอบเขตงาน ระยะเวลา วันสิ้นสุดบริการ ราคาประมาณ ใบเสนอราคา บรรทัดงบ · คำถามคัดกรอง 3 ข้อ</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>ATT-QUOTES · ATT-DPA</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>CONTRACT_WORK</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>จ้างเหมา</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>PURCHASE_REQUEST</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>งานเหมาช่วงที่มีงวดงาน เช่น เสาเข็ม โครงสร้างเหล็ก งานระบบ งานถนน</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>ขอบเขตงาน งวดงาน ไซต์ ราคาประมาณ บรรทัดงบ</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>ATT-QUOTES</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>IT_PURCHASE</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>ซื้ออุปกรณ์/ซอฟต์แวร์ไอที</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>PURCHASE_REQUEST</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>คอมพิวเตอร์ อุปกรณ์เครือข่าย ซอฟต์แวร์ และไลเซนส์</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>หมวด (HARDWARE/SOFTWARE) รายการ จำนวน ราคาประมาณ assetTag วันสิ้นสุดไลเซนส์ · คำถามคัดกรอง 3 ข้อ</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>ATT-QUOTES · ATT-DPA</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>NEW_SUPPLIER</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>ขอเพิ่มผู้ขายรายใหม่</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>SUPPLIER_REQUEST</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>ผู้ขายที่ยังไม่อยู่ในทะเบียน</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>ชื่อ เลขผู้เสียภาษี สาขา อีเมล เหตุผล</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -34406,7 +33733,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -35072,7 +34399,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -35363,7 +34690,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -35534,7 +34861,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -64696,7 +64023,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -69760,7 +69087,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -80879,7 +80206,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:J24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -81283,6 +80610,531 @@
       <c r="J10" t="inlineStr">
         <is>
           <t>เปลี่ยนผู้ดำรงตำแหน่ง ย้ายแผนก รักษาการแทน → กรรมการผู้จัดการ</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>1</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>BT-01</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>BUDGET_TRANSFER</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="7" t="n">
+        <v>100000</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>POSITION_OF_DEPARTMENT</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>8</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>โอนงบระหว่างบรรทัดไม่เกิน 100,000 → ผู้จัดการฝ่ายเจ้าของงบต้นทาง (ร่างระยะ 1 · รอลูกค้ายืนยัน OQ-40)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>1</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>BT-02</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>BUDGET_TRANSFER</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="n">
+        <v>100000</v>
+      </c>
+      <c r="E12" s="7" t="n">
+        <v>500000</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>POSITION_OF_DEPARTMENT</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>VP</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>8</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>โอนงบเกิน 100,000 ถึง 500,000 → รองกรรมการผู้จัดการสายงาน (ร่างระยะ 1 · รอลูกค้ายืนยัน OQ-40)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>1</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>BT-03</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>BUDGET_TRANSFER</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="n">
+        <v>500000</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>POSITION_OF_ORG</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>CFO</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>16</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>โอนงบเกิน 500,000 → CFO (ร่างระยะ 1 · รอลูกค้ายืนยัน OQ-40)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>1</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>OB-01</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>OVER_BUDGET</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>POSITION_OF_DEPARTMENT</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>VP</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>8</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>อนุมัติเกินงบไม่เกิน 50,000 → รองกรรมการผู้จัดการสายงาน (ร่างระยะ 1 · รอลูกค้ายืนยัน OQ-40)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>1</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>OB-02</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>OVER_BUDGET</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="E15" s="7" t="n">
+        <v>500000</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>POSITION_OF_ORG</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>CFO</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>16</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>อนุมัติเกินงบเกิน 50,000 ถึง 500,000 → CFO (ร่างระยะ 1 · รอลูกค้ายืนยัน OQ-40)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>1</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>OB-03</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>OVER_BUDGET</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="n">
+        <v>500000</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>POSITION_OF_ORG</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>16</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>อนุมัติเกินงบเกิน 500,000 → กรรมการผู้จัดการ (ร่างระยะ 1 · รอลูกค้ายืนยัน OQ-40)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>1</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>IE-01</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>INVOICE_EXCEPTION</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="7" t="n">
+        <v>20000</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>POSITION_OF_DEPARTMENT</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>8</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>ใบแจ้งหนี้ต่างจาก PO นอกเกณฑ์ ส่วนต่างไม่เกิน 20,000 → ผู้จัดการฝ่ายเจ้าของงบ (ร่างระยะ 1 · รอลูกค้ายืนยัน OQ-40)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>1</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>IE-02</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>INVOICE_EXCEPTION</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="n">
+        <v>20000</v>
+      </c>
+      <c r="E18" s="7" t="n">
+        <v>200000</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>POSITION_OF_DEPARTMENT</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>VP</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>8</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>ส่วนต่างเกิน 20,000 ถึง 200,000 → รองกรรมการผู้จัดการสายงาน (ร่างระยะ 1 · รอลูกค้ายืนยัน OQ-40)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>1</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>IE-03</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>INVOICE_EXCEPTION</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="n">
+        <v>200000</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>POSITION_OF_ORG</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>CFO</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>16</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>ส่วนต่างเกิน 200,000 → CFO (ร่างระยะ 1 · รอลูกค้ายืนยัน OQ-40)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>1</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>PC-01</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>PO_CHANGE</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" s="7" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>POSITION_OF_ORG</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>COO</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>8</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>แก้ PO ที่ยอดใหม่ไม่เกิน 1,000,000 → COO (ร่างระยะ 1 · รอลูกค้ายืนยัน OQ-40)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>1</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>PC-02</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>PO_CHANGE</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>POSITION_OF_ORG</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>16</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>แก้ PO ที่ยอดใหม่เกิน 1,000,000 → กรรมการผู้จัดการ (ร่างระยะ 1 · รอลูกค้ายืนยัน OQ-40)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>1</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>PAY-01</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>PAYMENT_RUN</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" s="7" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>POSITION_OF_ORG</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>CFO</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>8</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>รอบจ่ายไม่เกิน 5,000,000 → CFO (ผู้เตรียมห้ามอนุมัติ BR-SOD-04) (ร่างระยะ 1 · รอลูกค้ายืนยัน OQ-40)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>1</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>PAY-02</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>PAYMENT_RUN</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>POSITION_OF_ORG</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>16</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>รอบจ่ายเกิน 5,000,000 → กรรมการผู้จัดการ (ร่างระยะ 1 · รอลูกค้ายืนยัน OQ-40)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>1</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>BA-01</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>BANK_ACCOUNT_CHANGE</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>POSITION_OF_ORG</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>CFO</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>8</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>เพิ่มหรือเปลี่ยนบัญชีรับเงินของผู้ขาย → CFO (ผู้แก้ห้ามอนุมัติ BR-SOD-05) (ร่างระยะ 1 · รอลูกค้ายืนยัน OQ-40)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(workflow): S6-04 workflow version lifecycle, WF-SIMEC seed and validator
Draft, edit, dry-run, submit under DOA_CHANGE on subject WORKFLOW_VERSION with
step-up on the web only, publish and activation job; admin.workflow.*
capabilities; WF-SIMEC version 1 from sheet Workflow_Reviewers with
machine-readable conditions and fallbacks; spec rows §2.4 §10 §14.2.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/inputs/BCS_inputs_p1.xlsx
+++ b/docs/inputs/BCS_inputs_p1.xlsx
@@ -696,7 +696,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>ร่างผู้ตรวจคู่ขนานของระยะ 1 · seed ยังไม่อ่าน · S6 อ่านเอง</t>
+          <t>ผู้ตรวจคู่ขนานของระยะ 1 · seed สร้าง WF-SIMEC ฉบับ 1 จากชีตนี้ (S6)</t>
         </is>
       </c>
     </row>
@@ -807,7 +807,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -819,6 +819,9 @@
     <col width="18" customWidth="1" min="7" max="7"/>
     <col width="49" customWidth="1" min="8" max="8"/>
     <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -867,6 +870,21 @@
           <t>ref</t>
         </is>
       </c>
+      <c r="J1" s="6" t="inlineStr">
+        <is>
+          <t>whenJson</t>
+        </is>
+      </c>
+      <c r="K1" s="6" t="inlineStr">
+        <is>
+          <t>fallbackPosition</t>
+        </is>
+      </c>
+      <c r="L1" s="6" t="inlineStr">
+        <is>
+          <t>fallbackDepartment</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
@@ -914,6 +932,21 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="J2" s="5" t="inlineStr">
+        <is>
+          <t>เงื่อนไขแบบเครื่องอ่าน (JSON · {} = ทุกคำขอ)</t>
+        </is>
+      </c>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>ตำแหน่งผู้สำรอง</t>
+        </is>
+      </c>
+      <c r="L2" s="5" t="inlineStr">
+        <is>
+          <t>ฝ่ายของผู้สำรอง</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -959,6 +992,21 @@
           <t>FR-WF-101</t>
         </is>
       </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>VP</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>SUP</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1004,6 +1052,21 @@
           <t>FR-WF-101</t>
         </is>
       </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>{"field": "processesPersonalData", "op": "eq", "value": "Y"}</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>VP</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>SUP</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1049,6 +1112,21 @@
           <t>FR-WF-101</t>
         </is>
       </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>{"field": "$amountGross", "op": "gt", "value": "1000000.00"}</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>VP</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>SUP</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1094,6 +1172,21 @@
           <t>FR-WF-101</t>
         </is>
       </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>{"field": "$amountGross", "op": "gt", "value": "1000000.00"}</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>VP</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>OPS</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1139,6 +1232,21 @@
           <t>FR-WF-101</t>
         </is>
       </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>{"field": "$amountGross", "op": "gt", "value": "1000000.00"}</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>CFO</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>HQ</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1184,6 +1292,21 @@
           <t>FR-WF-101</t>
         </is>
       </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>{"field": "$lineCategories", "op": "anyIn", "value": ["SAFETY", "FUEL"]}</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>VP</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>OPS</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1227,6 +1350,21 @@
       <c r="I9" t="inlineStr">
         <is>
           <t>FR-WF-101</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>{"all": [{"field": "$budgetAccountCodes", "op": "anyIn", "value": ["121101", "121201", "121301"]}, {"field": "$amountGross", "op": "gt", "value": "500000.00"}]}</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>CFO</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>HQ</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(seed): S8-12 SIMEC plays every invoice scenario, supplier payment profiles, income types, S8 settings
- inputs_p1: RequestTypes retention columns (CONTRACT_WORK 500 bp, 365 days), S8 keys in Settings
  (matching wht ap numbering.AP numbering.WHT_CERT), validate_inputs checks them; make.py stays byte-stable
- seed/ap-profile.ts: SupplierPayment (payee type, default income type, credit days, e-Tax, registryFlag),
  WHT_Types (not yet confirmed), retention by request type, the S8 keys of Settings in org settings
- demo history: MATCH PRICE_WITHIN_TOL SERVICE_2WAY DUPLICATE ready; PRICE_OVER paid approved under
  INVOICE_EXCEPTION, others EXCEPTION; QTY_OVER short first receipt, paid rows get the rest and match
  again, others are closed short and stay EXCEPTION; MISSING without invoice; the inbox holds the second
  copy of each duplicate and one e-Tax invoice without a PO number

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/inputs/BCS_inputs_p1.xlsx
+++ b/docs/inputs/BCS_inputs_p1.xlsx
@@ -31003,7 +31003,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -31013,6 +31013,8 @@
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="32" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -31051,6 +31053,16 @@
           <t>active</t>
         </is>
       </c>
+      <c r="H1" s="6" t="inlineStr">
+        <is>
+          <t>defaultRetentionBp</t>
+        </is>
+      </c>
+      <c r="I1" s="6" t="inlineStr">
+        <is>
+          <t>defaultRetentionHoldDays</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
@@ -31088,6 +31100,16 @@
           <t>ใช้งาน (Y/N)</t>
         </is>
       </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>เงินประกันผลงานต่อใบ (basis point · 500 = 5% · S8)</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>ถือเงินประกันกี่วันหลังตรวจรับงวดสุดท้าย</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -31125,6 +31147,9 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -31162,6 +31187,9 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -31199,6 +31227,12 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="H5" t="n">
+        <v>500</v>
+      </c>
+      <c r="I5" t="n">
+        <v>365</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -31236,6 +31270,9 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -31272,6 +31309,9 @@
         <is>
           <t>Y</t>
         </is>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -33739,12 +33779,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="33" customWidth="1" min="2" max="2"/>
-    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
@@ -34075,320 +34115,534 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>priceAlertPct</t>
+          <t>matching.priceTolBp</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.1</v>
+        <v>100</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>เตือนเมื่อราคาใหม่แพงกว่าครั้งก่อนเกินเท่านี้</t>
+          <t>ราคาในใบแจ้งหนี้สูงกว่า PO ได้ไม่เกินกี่ basis point (100 = 1%)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>FR-P2P-003</t>
+          <t>OQ-121</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>digest.budgetLowPct</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>0.1</v>
+          <t>matching.priceTolAmount</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>1000.00</t>
+        </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>สรุปรายวันแจ้งบรรทัดงบที่เหลือต่ำกว่านี้</t>
+          <t>และไม่เกินกี่บาทต่อบรรทัด</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>FR-LINE-006</t>
+          <t>OQ-121</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>vatRounding</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>DOCUMENT</t>
-        </is>
+          <t>matching.qtyTolBp</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>0</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>คิด VAT ระดับเอกสาร</t>
+          <t>จำนวนในใบแจ้งหนี้เกินที่รับได้กี่ basis point</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>OQ-17</t>
+          <t>OQ-121</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>bahtTextStyle</t>
+          <t>matching.vatTolAmount</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>LIBREOFFICE</t>
+          <t>1.00</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>101 = หนึ่งร้อยหนึ่ง</t>
+          <t>VAT ในใบต่างจากที่คำนวณได้ไม่เกินกี่บาท</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>OQ-28</t>
+          <t>OQ-121</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>poWithoutPr</t>
+          <t>wht.minimumBase</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>1000.00</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ออก PO โดยไม่มี PR ได้ไหม</t>
+          <t>ไม่หักภาษี ณ ที่จ่ายเมื่อยอดก่อน VAT ของ PO ต่ำกว่านี้</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>OQ-24</t>
+          <t>OQ-122</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>newSupplierRequiresDoa</t>
+          <t>wht.timing</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>AT_PAYMENT</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>คำขอผู้ขายใหม่ต้องผ่าน DOA ไหม</t>
+          <t>หักภาษี ณ ที่จ่ายตอนจ่ายเงิน</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>OQ-23</t>
+          <t>OQ-122</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>printSignatureMode</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>APPROVAL_BLOCK</t>
-        </is>
+          <t>ap.defaultTermDays</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>30</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>เอกสารพิมพ์แสดงข้อมูลการอนุมัติแทนลายเซ็น</t>
+          <t>เครดิตตั้งต้นเมื่อ PO และผู้ขายไม่ระบุ (วัน)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>OQ-25</t>
+          <t>OQ-129</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>budgetCarryOver</t>
+          <t>ap.inboxAddress</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>ap@simec.bcs.local</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>ยกงบข้ามปีอัตโนมัติไหม</t>
+          <t>ที่อยู่กล่องรับใบแจ้งหนี้ทางอีเมล (สังเคราะห์)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>OQ-26</t>
+          <t>OQ-124</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>crossBudgetApproverDept</t>
+          <t>numbering.AP</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>CHARGED</t>
+          <t>AP-{BE}-{SEQ5}</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ใช้งบข้ามฝ่ายให้ผู้อนุมัติของฝ่ายเจ้าของงบ</t>
+          <t>รูปแบบเลขใบแจ้งหนี้ (ระบบออกตอนส่ง)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>OQ-27</t>
+          <t>OQ-12</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>email.fromAddress</t>
+          <t>numbering.WHT_CERT</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>no-reply@bcs.local</t>
+          <t>{BE}/{SEQ5}</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>ผู้ส่งอีเมล PO</t>
+          <t>รูปแบบเลขหนังสือรับรองการหักภาษี (50 ทวิ)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>OQ-22</t>
+          <t>OQ-12</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>retention.documentYears</t>
+          <t>priceAlertPct</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>5</v>
+        <v>0.1</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>เก็บเอกสารกี่ปี</t>
+          <t>เตือนเมื่อราคาใหม่แพงกว่าครั้งก่อนเกินเท่านี้</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>OQ-30</t>
+          <t>FR-P2P-003</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>line.channelOwner</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>BCS_DEMO</t>
-        </is>
+          <t>digest.budgetLowPct</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>0.1</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>ใช้ LINE OA ของ BCS จนกว่าลูกค้าจะมี OA (P0-04)</t>
+          <t>สรุปรายวันแจ้งบรรทัดงบที่เหลือต่ำกว่านี้</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>OQ-15 OQ-16</t>
+          <t>FR-LINE-006</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>express.encoding</t>
+          <t>vatRounding</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>UTF-8-BOM</t>
+          <t>DOCUMENT</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>encoding ไฟล์ส่ง Express (รอไฟล์ตัวอย่าง)</t>
+          <t>คิด VAT ระดับเอกสาร</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>OQ-10</t>
+          <t>OQ-17</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>poIdleDays</t>
-        </is>
-      </c>
-      <c r="B29" t="n">
-        <v>30</v>
+          <t>bahtTextStyle</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>LIBREOFFICE</t>
+        </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>PO ไม่มีความเคลื่อนไหวกี่วันจึงเตือนให้ปิด</t>
+          <t>101 = หนึ่งร้อยหนึ่ง</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>OQ-36</t>
+          <t>OQ-28</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t>poWithoutPr</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>ออก PO โดยไม่มี PR ได้ไหม</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>OQ-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>newSupplierRequiresDoa</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>คำขอผู้ขายใหม่ต้องผ่าน DOA ไหม</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>OQ-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>printSignatureMode</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>APPROVAL_BLOCK</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>เอกสารพิมพ์แสดงข้อมูลการอนุมัติแทนลายเซ็น</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>OQ-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>budgetCarryOver</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>ยกงบข้ามปีอัตโนมัติไหม</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>OQ-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>crossBudgetApproverDept</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>CHARGED</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>ใช้งบข้ามฝ่ายให้ผู้อนุมัติของฝ่ายเจ้าของงบ</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>OQ-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>email.fromAddress</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>no-reply@bcs.local</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>ผู้ส่งอีเมล PO</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>OQ-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>retention.documentYears</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>5</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>เก็บเอกสารกี่ปี</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>OQ-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>line.channelOwner</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>BCS_DEMO</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>ใช้ LINE OA ของ BCS จนกว่าลูกค้าจะมี OA (P0-04)</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>OQ-15 OQ-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>express.encoding</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>UTF-8-BOM</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>encoding ไฟล์ส่ง Express (รอไฟล์ตัวอย่าง)</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>OQ-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>poIdleDays</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>30</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>PO ไม่มีความเคลื่อนไหวกี่วันจึงเตือนให้ปิด</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>OQ-36</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
           <t>registry.mode</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B40" t="inlineStr">
         <is>
           <t>stub</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C40" t="inlineStr">
         <is>
           <t>ตรวจผู้ขายกับสรรพากรและ DBD: stub = ข้อมูลจำลอง</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D40" t="inlineStr">
         <is>
           <t>OQ-37</t>
         </is>

</xml_diff>

<commit_message>
test(e2e): P1-08 @p1demo mode and sheet Demo_Script_P1
- sheet Demo_Script_P1 in the phase-1 workbook (scripts/inputs_p1/p1_demo.py): 16 scenes, 14 core, rows verified
  against the code and the seeded data
- p1demo mode: `pnpm test:e2e --grep @p1demo` seeds SIMEC from the phase-1 workbook on bcs_e2e_p1demo, project
  p1demo runs tests/e2e/p1demo/*.spec.ts in file order; verify --e2e runs it after @demo and merges the reports
- tests/e2e/p1demo/support.ts reads the sheet; 00-sheet.spec.ts holds the sheet and the scene files together;
  the demo day script reads the phase-1 workbook in this mode

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/inputs/BCS_inputs_p1.xlsx
+++ b/docs/inputs/BCS_inputs_p1.xlsx
@@ -33,6 +33,7 @@
     <sheet name="Request_History" sheetId="24" state="visible" r:id="rId24"/>
     <sheet name="DocSamples" sheetId="25" state="visible" r:id="rId25"/>
     <sheet name="Scenarios" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="Demo_Script_P1" sheetId="27" state="visible" r:id="rId27"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -489,7 +490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:B27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -793,6 +794,18 @@
       <c r="B26" s="2" t="inlineStr">
         <is>
           <t>ตำแหน่งของสถานการณ์ทดสอบที่ฝังในข้อมูล เช่น แตกยอด คำขอซ้ำ งานค้าง งบใกล้หมด ผู้ขายเลิกกิจการ</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Demo_Script_P1</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>ฉาก demo ระยะ 1 เรียงตามลำดับของวัน (P1-08): ผู้ทำ ยอด เอกสารที่ใช้ และผลที่คาด · e2e @p1demo อ่านชีตนี้เอง ทุกฉาก core = Y ต้องผ่าน</t>
         </is>
       </c>
     </row>
@@ -70567,6 +70580,1998 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:AF18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="29" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="20" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="23" customWidth="1" min="16" max="16"/>
+    <col width="13" customWidth="1" min="17" max="17"/>
+    <col width="10" customWidth="1" min="18" max="18"/>
+    <col width="11" customWidth="1" min="19" max="19"/>
+    <col width="32" customWidth="1" min="20" max="20"/>
+    <col width="24" customWidth="1" min="21" max="21"/>
+    <col width="27" customWidth="1" min="22" max="22"/>
+    <col width="32" customWidth="1" min="23" max="23"/>
+    <col width="17" customWidth="1" min="24" max="24"/>
+    <col width="16" customWidth="1" min="25" max="25"/>
+    <col width="18" customWidth="1" min="26" max="26"/>
+    <col width="44" customWidth="1" min="27" max="27"/>
+    <col width="15" customWidth="1" min="28" max="28"/>
+    <col width="13" customWidth="1" min="29" max="29"/>
+    <col width="60" customWidth="1" min="30" max="30"/>
+    <col width="20" customWidth="1" min="31" max="31"/>
+    <col width="60" customWidth="1" min="32" max="32"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>scene</t>
+        </is>
+      </c>
+      <c r="B1" s="9" t="inlineStr">
+        <is>
+          <t>core</t>
+        </is>
+      </c>
+      <c r="C1" s="9" t="inlineStr">
+        <is>
+          <t>stage</t>
+        </is>
+      </c>
+      <c r="D1" s="9" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="E1" s="9" t="inlineStr">
+        <is>
+          <t>titleTh</t>
+        </is>
+      </c>
+      <c r="F1" s="9" t="inlineStr">
+        <is>
+          <t>actor</t>
+        </is>
+      </c>
+      <c r="G1" s="9" t="inlineStr">
+        <is>
+          <t>others</t>
+        </is>
+      </c>
+      <c r="H1" s="9" t="inlineStr">
+        <is>
+          <t>channel</t>
+        </is>
+      </c>
+      <c r="I1" s="9" t="inlineStr">
+        <is>
+          <t>requestType</t>
+        </is>
+      </c>
+      <c r="J1" s="9" t="inlineStr">
+        <is>
+          <t>chargedDept</t>
+        </is>
+      </c>
+      <c r="K1" s="9" t="inlineStr">
+        <is>
+          <t>budgetKey</t>
+        </is>
+      </c>
+      <c r="L1" s="9" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="M1" s="9" t="inlineStr">
+        <is>
+          <t>supplier</t>
+        </is>
+      </c>
+      <c r="N1" s="9" t="inlineStr">
+        <is>
+          <t>itemCode</t>
+        </is>
+      </c>
+      <c r="O1" s="9" t="inlineStr">
+        <is>
+          <t>qty</t>
+        </is>
+      </c>
+      <c r="P1" s="9" t="inlineStr">
+        <is>
+          <t>unitPrice</t>
+        </is>
+      </c>
+      <c r="Q1" s="9" t="inlineStr">
+        <is>
+          <t>net</t>
+        </is>
+      </c>
+      <c r="R1" s="9" t="inlineStr">
+        <is>
+          <t>vat</t>
+        </is>
+      </c>
+      <c r="S1" s="9" t="inlineStr">
+        <is>
+          <t>gross</t>
+        </is>
+      </c>
+      <c r="T1" s="9" t="inlineStr">
+        <is>
+          <t>historyRef</t>
+        </is>
+      </c>
+      <c r="U1" s="9" t="inlineStr">
+        <is>
+          <t>docSample</t>
+        </is>
+      </c>
+      <c r="V1" s="9" t="inlineStr">
+        <is>
+          <t>invoiceNo</t>
+        </is>
+      </c>
+      <c r="W1" s="9" t="inlineStr">
+        <is>
+          <t>invoiceUnitPrice</t>
+        </is>
+      </c>
+      <c r="X1" s="9" t="inlineStr">
+        <is>
+          <t>expectedOutcome</t>
+        </is>
+      </c>
+      <c r="Y1" s="9" t="inlineStr">
+        <is>
+          <t>expectedRule</t>
+        </is>
+      </c>
+      <c r="Z1" s="9" t="inlineStr">
+        <is>
+          <t>expectedApprover</t>
+        </is>
+      </c>
+      <c r="AA1" s="9" t="inlineStr">
+        <is>
+          <t>expectedReviewers</t>
+        </is>
+      </c>
+      <c r="AB1" s="9" t="inlineStr">
+        <is>
+          <t>escalated</t>
+        </is>
+      </c>
+      <c r="AC1" s="9" t="inlineStr">
+        <is>
+          <t>delegation</t>
+        </is>
+      </c>
+      <c r="AD1" s="9" t="inlineStr">
+        <is>
+          <t>expectJson</t>
+        </is>
+      </c>
+      <c r="AE1" s="9" t="inlineStr">
+        <is>
+          <t>minutes</t>
+        </is>
+      </c>
+      <c r="AF1" s="9" t="inlineStr">
+        <is>
+          <t>stepsTh</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>ฉาก (= เลขไฟล์ e2e)</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Y = ต้องผ่านก่อนเส้นชัย A3</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>ขั้นเจ้าของฉาก</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>หัวข้อตามรายการใน P1-08</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>หัวข้อที่พูดตอน demo</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>ผู้ทำ (ชีต Users)</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>ผู้ใช้อื่นที่ลงมือในฉาก คั่นด้วย ·</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>WEB LIFF LINE_CHAT APP APP_OFFLINE EMAIL</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>ประเภทคำขอ</t>
+        </is>
+      </c>
+      <c r="J2" s="5" t="inlineStr">
+        <is>
+          <t>แผนกเจ้าของงบ</t>
+        </is>
+      </c>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>กุญแจงบ (ปีงบตามวันที่เล่น)</t>
+        </is>
+      </c>
+      <c r="L2" s="5" t="inlineStr">
+        <is>
+          <t>สถานที่ส่ง</t>
+        </is>
+      </c>
+      <c r="M2" s="5" t="inlineStr">
+        <is>
+          <t>ผู้ขาย</t>
+        </is>
+      </c>
+      <c r="N2" s="5" t="inlineStr">
+        <is>
+          <t>รายการ (ชีต Items)</t>
+        </is>
+      </c>
+      <c r="O2" s="5" t="inlineStr">
+        <is>
+          <t>จำนวน</t>
+        </is>
+      </c>
+      <c r="P2" s="5" t="inlineStr">
+        <is>
+          <t>ราคาต่อหน่วย ก่อน VAT</t>
+        </is>
+      </c>
+      <c r="Q2" s="5" t="inlineStr">
+        <is>
+          <t>ยอดก่อน VAT</t>
+        </is>
+      </c>
+      <c r="R2" s="5" t="inlineStr">
+        <is>
+          <t>VAT</t>
+        </is>
+      </c>
+      <c r="S2" s="5" t="inlineStr">
+        <is>
+          <t>รวม VAT</t>
+        </is>
+      </c>
+      <c r="T2" s="5" t="inlineStr">
+        <is>
+          <t>คำขอใน Request_History ที่ฉากใช้</t>
+        </is>
+      </c>
+      <c r="U2" s="5" t="inlineStr">
+        <is>
+          <t>เอกสารในชีต DocSamples</t>
+        </is>
+      </c>
+      <c r="V2" s="5" t="inlineStr">
+        <is>
+          <t>เลขที่ใบแจ้งหนี้ของผู้ขาย</t>
+        </is>
+      </c>
+      <c r="W2" s="5" t="inlineStr">
+        <is>
+          <t>ราคาต่อหน่วยในใบแจ้งหนี้ ก่อน VAT</t>
+        </is>
+      </c>
+      <c r="X2" s="5" t="inlineStr">
+        <is>
+          <t>ผลที่คาด</t>
+        </is>
+      </c>
+      <c r="Y2" s="5" t="inlineStr">
+        <is>
+          <t>ข้อ DOA ที่คาด</t>
+        </is>
+      </c>
+      <c r="Z2" s="5" t="inlineStr">
+        <is>
+          <t>ผู้อนุมัติที่คาด</t>
+        </is>
+      </c>
+      <c r="AA2" s="5" t="inlineStr">
+        <is>
+          <t>ผู้ตรวจคู่ขนานที่คาด ข้อ=ผู้ใช้ คั่นด้วย ·</t>
+        </is>
+      </c>
+      <c r="AB2" s="5" t="inlineStr">
+        <is>
+          <t>ยกระดับ (Y/N)</t>
+        </is>
+      </c>
+      <c r="AC2" s="5" t="inlineStr">
+        <is>
+          <t>รักษาการแทน</t>
+        </is>
+      </c>
+      <c r="AD2" s="5" t="inlineStr">
+        <is>
+          <t>ค่าที่คาดเฉพาะเรื่อง (JSON)</t>
+        </is>
+      </c>
+      <c r="AE2" s="5" t="inlineStr">
+        <is>
+          <t>นาทีที่ใช้ตอน demo</t>
+        </is>
+      </c>
+      <c r="AF2" s="5" t="inlineStr">
+        <is>
+          <t>ลำดับคลิกโดยย่อ (runbook ของ P1-12 ขยาย)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>S6</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>PARALLEL_REVIEW</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>ขอจ้างเหมางานถนนช่วงที่ 2 ผ่านผู้ตรวจ 3 ฝ่ายพร้อมกัน</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>pm_p07</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>dm_qse · dm_leg · dm_fin</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>WEB</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>CONTRACT_WORK</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>CONI</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>P07-SUB</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>SITE-P07</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>SP0105</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>SUB-010</t>
+        </is>
+      </c>
+      <c r="O3" t="n">
+        <v>8000</v>
+      </c>
+      <c r="P3" s="7" t="n">
+        <v>260</v>
+      </c>
+      <c r="Q3" s="7" t="n">
+        <v>2080000</v>
+      </c>
+      <c r="R3" s="7" t="n">
+        <v>145600</v>
+      </c>
+      <c r="S3" s="7" t="n">
+        <v>2225600</v>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>ROUTED</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>PR-03</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>ceo</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>RV-03=dm_leg · RV-04=dm_qse · RV-05=dm_fin</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>{"requestTitleTh":"งานถนนแอสฟัลต์ช่วงที่ 2 (ค่าแรงและเครื่องจักร) 8,000 ตร.ม. · ถนนเลี่ยงเมืองราชบุรี","form":{"scopeOfWork":"งานถนนแอสฟัลต์ช่วงที่ 2 (ค่าแรงและเครื่องจักร) ตามแบบและรายการประกอบแบบ","milestones":"งวดที่ 1 30% เมื่อเริ่มงานและส่งแผนงาน · งวดที่ 2 40% เมื่องานเสร็จ 70% · งวดที่ 3 30% เมื่อส่งมอบงาน (หักประกันผลงาน 5%)","site":"หน้างานโครงการ P07 ถนนเลี่ยงเมืองราชบุรี"},"lineFromCatalog":true,"quotes":[{"supplier":"SP0105","amount":"2080000.00","includesVat":false,"chosen":true}],"singleSourceReasonTh":"ผู้รับเหมารายเดิมของงานถนนช่วงที่ 1 มีเครื่องจักรอยู่หน้างานแล้ว ราคาต่อหน่วยเท่าสัญญาเดิม","preSendRoute":{"rule":"PR-03","approver":"ceo","showsReviewers":false},"reviewMode":"ALL","reviewSlaHours":16,"reviewDecisions":[{"member":"dm_qse","rule":"RV-04","channel":"LINE_CHAT","decision":"PASS"},{"member":"dm_leg","rule":"RV-03","channel":"WEB","decision":"ASK_INFO_THEN_PASS","questionTh":"ขอร่างสัญญาจ้างเหมาช่วงที่ 2 และหลักประกันสัญญาก่อนตรวจ","answerTh":"ใช้ร่างสัญญาแบบเดียวกับช่วงที่ 1 หลักประกันผลงาน 5% ตามงวดงาน"},{"member":"dm_fin","rule":"RV-05","channel":"WEB","decision":"PASS"}],"afterReviews":{"stepNo":2,"rule":"PR-03","approver":"ceo","stepUp":true,"taskOpen":true},"flags":[],"notDuplicateOf":"H229","priceRef":{"item":"SUB-010","count":2,"median":"260.00","status":"FEW_SAMPLES"}}</t>
+        </is>
+      </c>
+      <c r="AE3" t="n">
+        <v>6</v>
+      </c>
+      <c r="AF3" t="inlineStr">
+        <is>
+          <t>pm_p07 เข้าระบบ → ขอซื้อ / ขอจ้าง → จ้างเหมา → กรอกชื่อคำขอ ขอบเขตงาน งวดงาน ไซต์งาน → รายการที่ 1 เลือก SUB-010 จากแคตตาล็อก 8,000 ตร.ม. × 260.00 บนบรรทัดงบ P07-SUB สถานที่ส่ง SITE-P07 → ผู้ขาย SP0105 แนบใบเสนอราคา 1 ใบ ใส่เหตุผลกรณีมีผู้ขายรายเดียว → ตรวจและส่ง (เส้นทางที่คาด: DOA-SIMEC ฉบับ 1 ข้อ PR-03 ceo) → ส่งขออนุมัติ → หน้าคำขอ: ขั้นที่ 1 · ผู้ตรวจ ผ่านแล้ว 0 ใน 3 ฝ่าย → dm_qse กด ผ่าน ในการ์ด LINE → dm_leg ขอข้อมูลเพิ่ม → pm_p07 ตอบ → dm_leg กด ผ่าน → dm_fin กด ผ่าน บนเว็บ → ผ่านแล้ว 3 ใน 3 ฝ่าย งานไปรอที่ ceo</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>S17</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>APP_APPROVE</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>ceo อนุมัติงานถนนช่วงที่ 2 ในแอป BCS Go ด้วยลายนิ้วมือ</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>ceo</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>APP</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>PR-03</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>ceo</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>{"requestOfScene":1,"push":true,"pushTemplate":"task.assigned","passkeyDeviceLabel":"โทรศัพท์ของ CEO","stepUpMethod":"PASSKEY","decisionChannel":"APP","requestStatusAfter":"APPROVED"}</t>
+        </is>
+      </c>
+      <c r="AE4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>ก่อนวัน demo: ceo ลงทะเบียน passkey ในแอป (ตั้งค่าของฉัน → PIN ยืนยันธุรกรรม → เพิ่ม passkey บนเครื่องนี้ → ใส่รหัสผ่านและชื่อเครื่อง → ยืนยันและเพิ่ม passkey → สแกนนิ้ว) และเปิดรับแจ้งเตือนในแอป · ระหว่าง demo: งานถนนช่วงที่ 2 ของฉาก 1 ผ่านผู้ตรวจครบ 3 ฝ่าย → มือถือ ceo ได้แจ้งเตือน "มีงานรออนุมัติ" เนื้อความเป็นเลข PR อย่างเดียว (ไม่มียอด ชื่อ หรือชื่อเรื่อง) → แตะเปิดงานในแอป → อนุมัติ → ยอดตั้งแต่ 100,000 บาทจึงต้องยืนยัน → อนุมัติด้วยลายนิ้วมือหรือใบหน้า (passkey) → สแกนนิ้ว → เห็น "อนุมัติแล้ว" → เปิดหน้าคำขอ: เส้นทางอนุมัติและแท็บประวัติแสดงช่องทาง "แอป BCS Go" ข้างการอนุมัติของ ceo</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>S6</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>WORKFLOW_TRYOUT</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>ลดเกณฑ์ผู้ตรวจงานจ้างเหมา ทดลองเส้นทางก่อนส่งเผยแพร่</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>admin2</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>ceo</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>WEB</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>CONTRACT_WORK</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>CONI</t>
+        </is>
+      </c>
+      <c r="S5" s="7" t="n">
+        <v>800000</v>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>DOA-CHG-01</t>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>ceo</t>
+        </is>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>{"workflowCode":"WF-SIMEC","fromVersion":1,"draftVersion":2,"rules":7,"draftRules":[{"rule":"RV-03","field":"$amountGross","op":"gt","from":"1000000.00","to":"500000.00"},{"rule":"RV-04","field":"$amountGross","op":"gt","from":"1000000.00","to":"500000.00"},{"rule":"RV-05","field":"$amountGross","op":"gt","from":"1000000.00","to":"500000.00"}],"changeReasonTh":"ลดเกณฑ์ผู้ตรวจงานจ้างเหมาเป็นยอดรวม VAT เกิน 500,000 บาท","effectiveDate":"DEFAULT_FIRST_OF_NEXT_MONTH","dryRun":{"requestType":"CONTRACT_WORK","amountGross":"800000.00","requester":"pm_p07","department":"CONI"},"liveReviewers":[],"draftReviewers":["RV-03=dm_leg","RV-04=dm_qse","RV-05=dm_fin"],"doaRule":"PR-03","doaApprover":"ceo","backtest":{"windowDays":90,"changed":1,"refs":["H149"]},"approvalRule":"DOA-CHG-01","approver":"ceo","pin":true,"afterApproval":{"v1":"IN_EFFECT","v2":"UPCOMING"},"changesLaterScenes":false}</t>
+        </is>
+      </c>
+      <c r="AE5" t="n">
+        <v>6</v>
+      </c>
+      <c r="AF5" t="inlineStr">
+        <is>
+          <t>admin2 เข้าระบบ → ผู้ตรวจคู่ขนาน (workflow) → สร้างร่างจาก WF-SIMEC ฉบับ 1 → แก้ข้อ RV-03 RV-04 RV-05 เป็นยอดรวม VAT มากกว่า 500,000.00 → ใส่เหตุผลที่เปลี่ยน แล้วบันทึกร่าง → แท็บทดลองส่ง: จ้างเหมา ยอดรวม VAT 800,000.00 ผู้ขอ pm_p07 → ฉบับที่มีผลไม่มีผู้ตรวจ ร่างมีผู้ตรวจ 3 ฝ่าย → ย้อนทดสอบ 90 วัน เปลี่ยนเส้นทาง 1 ฉบับ → ตรวจและส่งขออนุมัติเผยแพร่ → ceo เปิดงาน ใส่ PIN อนุมัติการเปลี่ยนนี้ → ฉบับ 2 อนุมัติแล้ว รอมีผล ฉบับ 1 ยังมีผลอยู่</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>S6</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>BUDGET_TRANSFER</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>โอนงบเช่าเครื่องจักรไปงบจ้างเหมา โครงการ P07</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>fin_bud1</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>vp_ops</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>WEB</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>CONI</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>P07-RENT</t>
+        </is>
+      </c>
+      <c r="Q6" s="7" t="n">
+        <v>300000</v>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>BT-02</t>
+        </is>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>vp_ops</t>
+        </is>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>{"kind":"TRANSFER","fromKey":"P07-RENT","toKey":"P07-SUB","amount":"300000.00","reasonTh":"ย้ายงบเช่าเครื่องจักรที่ยังไม่ใช้ไปงบจ้างเหมางานถนนช่วงที่ 2","rule":"BT-02","approver":"vp_ops","pin":true,"plannedFrom":"SHEET_BUDGET_OF_RUN_FY","dashboard":{"from":{"transferredOut":"300000.00","currentIsPlannedMinusAmount":true},"to":{"transferredIn":"300000.00","currentIsPlannedPlusAmount":true}},"events":["budget_transfer.drafted","budget_transfer.submitted","approval_task.decided","budget_transfer.approved"]}</t>
+        </is>
+      </c>
+      <c r="AE6" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF6" t="inlineStr">
+        <is>
+          <t>fin_bud1 เข้าระบบ → งบประมาณ → การโอนและปรับงบ → โอนหรือปรับงบ → โอนระหว่างบรรทัด จาก P07-RENT ไป P07-SUB ของปีงบนี้ 300,000.00 ใส่เหตุผล → ส่งขออนุมัติ (ข้อ BT-02 รอ vp_ops) → vp_ops เปิดงาน อนุมัติ ใส่ PIN → fin_bud1 เปิดหน้างบประมาณ กดที่มาของงบ เห็นงบตั้งต้น โอนออก โอนเข้า และงบปัจจุบันของทั้งสองบรรทัด</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>S6</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>DUPLICATE</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>ส่งคำขอลวดผูกเหล็กซ้ำ ระบบให้บอกเหตุผลก่อนส่ง</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>se_p06a</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>vp_ops</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>WEB</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>BUY_GOODS</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>CONI</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>P06-MAT</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>SITE-P06</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>SP0016</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>MAT-014</t>
+        </is>
+      </c>
+      <c r="O7" t="n">
+        <v>500</v>
+      </c>
+      <c r="P7" s="7" t="n">
+        <v>62</v>
+      </c>
+      <c r="Q7" s="7" t="n">
+        <v>31000</v>
+      </c>
+      <c r="R7" s="7" t="n">
+        <v>2170</v>
+      </c>
+      <c r="S7" s="7" t="n">
+        <v>33170</v>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>ROUTED</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>PR-02</t>
+        </is>
+      </c>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t>vp_ops</t>
+        </is>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>{"requestTitleTh":"ลวดผูกเหล็ก 500 กก. งานตอม่อ · สะพานข้ามแยกลำลูกกา","sendTimes":2,"secondHow":"REORDER","lineFromCatalog":true,"firstFlags":[],"flag":"DUPLICATE","refusalReason":"DUPLICATE_UNACKNOWLEDGED","reasonTh":"ลวดชุดแรกใช้ผูกเหล็กคานสะพานหมดแล้ว ชุดนี้สำหรับงานตอม่อ","windowDays":7,"historyPairOutsideWindow":["H169","H171"],"noSplitWith":["H240"],"approverSees":{"badgeTh":"คล้ายคำขอที่ส่งไปแล้ว","reasonPrefixTh":"เหตุผลของผู้ขอ: "}}</t>
+        </is>
+      </c>
+      <c r="AE7" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF7" t="inlineStr">
+        <is>
+          <t>se_p06a เข้าระบบ → ขอซื้อ / ขอจ้าง → ซื้อของ → ลวดผูกเหล็ก MAT-014 จากแคตตาล็อก 500 กก. × 62.00 บนงบ P06-MAT สถานที่ส่ง SITE-P06 ผู้ขาย SP0016 → ส่งขออนุมัติ (ไม่มีเตือน รอ vp_ops) → หน้าคำขอ กด ขอซ้ำ → ตรวจและส่ง → ระบบเตือน คำขอนี้คล้ายคำขอที่คุณส่งไปแล้ว พร้อมลิงก์ใบแรก → กดส่งโดยไม่ใส่เหตุผลไม่ได้ → ใส่เหตุผลที่ขออีกครั้ง แล้วส่ง → vp_ops เปิดงาน เห็นป้าย คล้ายคำขอที่ส่งไปแล้ว และเหตุผลของผู้ขอ</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>S6</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>OVER_BUDGET</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>ขอจัดงานเปิดตัวโครงการบนงบการตลาดที่เหลือไม่ถึง 10%</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>mkt_01</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>cfo</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>WEB</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>HIRE_SERVICE</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>MKT</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>MKT-OPEX</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>HQ-STORE</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>SP0182</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>MKT-004</t>
+        </is>
+      </c>
+      <c r="O8" t="n">
+        <v>1</v>
+      </c>
+      <c r="P8" s="7" t="n">
+        <v>185000</v>
+      </c>
+      <c r="Q8" s="7" t="n">
+        <v>185000</v>
+      </c>
+      <c r="R8" s="7" t="n">
+        <v>12950</v>
+      </c>
+      <c r="S8" s="7" t="n">
+        <v>197950</v>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>ROUTED</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>OB-02</t>
+        </is>
+      </c>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t>cfo</t>
+        </is>
+      </c>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t>{"requestTitleTh":"ค่าจัดงานเปิดตัวโครงการใหม่ · ฝ่ายการตลาดและลูกค้าสัมพันธ์","form":{"scopeOfWork":"ค่าจัดงานเปิดตัวโครงการใหม่ ที่คลังสำนักงานใหญ่","servicePeriod":"1 ครั้ง","processesPersonalData":"N","accessesSystems":"N","accessesPremises":"Y"},"serviceEndInDays":30,"quotes":[{"supplier":"SP0182","amount":"185000.00","chosen":true},{"supplier":"ผู้เสนอราคาเปรียบเทียบ 1","amount":"192400.00"},{"supplier":"ผู้เสนอราคาเปรียบเทียบ 2","amount":"197950.00"}],"draftBy":"SCENE_SCRIPT","lowPct":10,"firstSubmit":"BUDGET_INSUFFICIENT","overrunRule":"OB-02","overrunApprover":"cfo","overrunPin":false,"reasonTh":"งานเปิดตัวโครงการใหม่ต้องจัดในไตรมาสนี้","requestRule":"PR-03","requestApprover":"ceo","availableAfterSend":"0.00"}</t>
+        </is>
+      </c>
+      <c r="AE8" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF8" t="inlineStr">
+        <is>
+          <t>mkt_01 เข้าระบบ เปิดร่างค่าจัดงานเปิดตัวโครงการ 185,000.00 บนงบ MKT-OPEX → หน้าคำขอบอก งบไม่พอ คงเหลือ 96,000.00 ขาดอีก 89,000.00 → กด ขออนุมัติเกินงบ ใส่เหตุผล → ส่ง (ข้อ OB-02 รอ cfo) → cfo เปิดงาน อนุมัติ → mkt_01 เปิดคำขอ ตรวจและส่ง → ส่งขออนุมัติแล้ว รอ ceo (ข้อ PR-03)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>S17</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>OFFLINE_RECEIVE</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>ตรวจรับคอนกรีตผสมเสร็จที่หน้างาน P07 ตอนไม่มีสัญญาณ</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>store_p07</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>APP_OFFLINE</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>BUY_GOODS</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>CONI</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>P07-MAT</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>SITE-P07</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>SP0039</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>RMC-004</t>
+        </is>
+      </c>
+      <c r="O9" t="n">
+        <v>2</v>
+      </c>
+      <c r="P9" s="7" t="n">
+        <v>2780</v>
+      </c>
+      <c r="Q9" s="7" t="n">
+        <v>5560</v>
+      </c>
+      <c r="R9" s="7" t="n">
+        <v>389.2</v>
+      </c>
+      <c r="S9" s="7" t="n">
+        <v>5949.2</v>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>H042</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>RECEIVED</t>
+        </is>
+      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>{"find":"TYPED","deliveryNoteNo":"DN-RMC-0716","photos":1,"lostAnswers":1,"poStatusBefore":"SENT","poStatusAfter":"RECEIVED","receipts":1,"receiptStatus":"POSTED","receiptChannel":"APP","offline":true}</t>
+        </is>
+      </c>
+      <c r="AE9" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF9" t="inlineStr">
+        <is>
+          <t>ตอนมีสัญญาณ store_p07 เปิดแอป BCS Go → เมนู ตรวจรับ → ตรวจรับหน้างานแบบไม่มีสัญญาณ (BCS Go) → เตรียมตรวจรับออฟไลน์ (เห็น PO คอนกรีตผสมเสร็จ 400 กก./ตร.ซม. ในรายการ) → ปิดสัญญาณ → สแกน QR บน PO หรือพิมพ์เลขใบสั่งซื้อ → หาใบสั่งซื้อ → บันทึกตรวจรับ → รับรอบนี้ 2 ลบ.ม. · เลขที่ใบส่งของ · ถ่ายรูปของที่มาส่ง → บันทึกไว้ในเครื่อง → เห็น "บันทึกไว้ในเครื่องแล้ว จะส่งให้เองเมื่อมีสัญญาณ" และ รอส่ง 1 → เปิดสัญญาณ → หน้าอัปโหลดรูปแล้วส่งเอง → "ไม่มีรายการค้างในเครื่อง" → บนเว็บ PO เป็น รับครบแล้ว มี GR 1 ใบพร้อมรูป · ฉาก e2e จำลองคำตอบที่หายหนึ่งครั้ง: หน้าส่งซ้ำด้วยรหัสเดิม ได้ผลเดิม GR ใบเดียว</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>S8</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>INVOICE_EMAIL</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>ใบกำกับภาษีอิเล็กทรอนิกส์ของเหล็กข้ออ้อยมาทางอีเมล ตรง 3 ทางแล้วพร้อมจ่าย</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>fin_ap1</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>EMAIL</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>BUY_GOODS</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>CONI</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>P07-MAT</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>SITE-P07</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>SP0029</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>STL-004</t>
+        </is>
+      </c>
+      <c r="O10" t="n">
+        <v>4</v>
+      </c>
+      <c r="P10" s="7" t="n">
+        <v>23500</v>
+      </c>
+      <c r="Q10" s="7" t="n">
+        <v>94000</v>
+      </c>
+      <c r="R10" s="7" t="n">
+        <v>6580</v>
+      </c>
+      <c r="S10" s="7" t="n">
+        <v>100580</v>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>H144</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>S00276/A</t>
+        </is>
+      </c>
+      <c r="W10" s="7" t="n">
+        <v>23500</v>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>MATCHED</t>
+        </is>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>{"invoiceDate":"RUN_DATE","dueAfterDays":30,"mail":{"from":"SUPPLIER_EMAIL","to":"SETTING:ap.inboxAddress","subjectTh":"ใบแจ้งหนี้ {invoiceNo} ตาม {poNumber}","attachment":"ETAX_XML","clearMailboxFirst":true},"poll":{"received":1,"drafts":1,"failed":0},"draft":{"channel":"EMAIL","prefill":"ETAX_XML","statedVat":"6580.00"},"accountCode":"510101","costCenter":"CC-P07","matchResult":"MATCHED","status":"READY_FOR_PAYMENT","payable":"100580.00","expectedWht":"0.00","expectedTransfer":"100580.00","budget":{"committed":"-94000.00","actual":"94000.00","available":"0.00"},"events":["inbound_email.received","inbound_email.processed","invoice.drafted","invoice.coding_confirmed","invoice.submitted","invoice.matched","invoice.ready","budget.actualized"]}</t>
+        </is>
+      </c>
+      <c r="AE10" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF10" t="inlineStr">
+        <is>
+          <t>ก่อนฉาก สคริปต์ส่งอีเมลของผู้ขาย SP0029 แนบใบกำกับภาษีอิเล็กทรอนิกส์ (XML) เลขที่ S00276/A อ้าง PO ของ H144 ไปที่กล่องรับขององค์กร → fin_ap1 เมนู ใบแจ้งหนี้ → กล่องรับใบแจ้งหนี้ → ดึงอีเมลตอนนี้ (อีเมลใหม่ 1 ฉบับ สร้างร่าง 1 ใบ) → เปิด ใบแจ้งหนี้ S00276/A · ร่าง → ชี้ป้าย จาก e-Tax ที่เลขที่ วันที่ และ VAT กับผู้ขายและ PO ที่ระบบเลือกให้ → ยืนยันรหัสบัญชีทุกบรรทัด → ส่งจับคู่ → ตรงทุกบรรทัด พร้อมจ่าย ครบกำหนดอีก 30 วัน → เปิดงบ P07-MAT เห็นผูกพันลดและใช้จริงเพิ่ม 94,000.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>S8</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>INVOICE_UPLOAD</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>อัปโหลดใบแจ้งหนี้เบรกเกอร์ที่ราคาเกิน PO แล้วขออนุมัติส่วนต่างตาม DOA</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>fin_ap2</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>proc_officer · dm_mep</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>WEB</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>BUY_GOODS</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>MEP</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>MEP-OPEX</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>HQ-STORE</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>SP0044</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>ELE-006</t>
+        </is>
+      </c>
+      <c r="O11" t="n">
+        <v>18</v>
+      </c>
+      <c r="P11" s="7" t="n">
+        <v>3200</v>
+      </c>
+      <c r="Q11" s="7" t="n">
+        <v>57600</v>
+      </c>
+      <c r="R11" s="7" t="n">
+        <v>4032</v>
+      </c>
+      <c r="S11" s="7" t="n">
+        <v>61632</v>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>H074</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>S00829/A</t>
+        </is>
+      </c>
+      <c r="W11" s="7" t="n">
+        <v>3300</v>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>EXCEPTION</t>
+        </is>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>IE-01</t>
+        </is>
+      </c>
+      <c r="Z11" t="inlineStr">
+        <is>
+          <t>dm_mep</t>
+        </is>
+      </c>
+      <c r="AB11" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>{"invoiceDate":"RUN_DATE","dueAfterDays":30,"file":"PDF","draft":{"channel":"UPLOAD","prefill":"MANUAL"},"invoiceNet":"59400.00","invoiceVat":"4158.00","invoiceGross":"63558.00","accountCode":"530301","costCenter":"CC-MEP","matchResult":"EXCEPTION","exceptionType":"PRICE_OVER","exceptionAssignee":"PROCUREMENT","variance":"1800.00","varianceVat":"126.00","varianceGross":"1926.00","varianceBy":"proc_officer","varianceReasonTh":"ผู้ผลิตปรับราคาเบรกเกอร์ขึ้นตามประกาศ","varianceRule":"IE-01","varianceApprover":"dm_mep","stepUp":false,"status":"READY_FOR_PAYMENT","payable":"63558.00","expectedWht":"0.00","budget":{"committed":"-57600.00","actual":"59400.00","available":"-1800.00"},"events":["invoice.drafted","invoice.coding_confirmed","invoice.submitted","invoice.exception_raised","invoice.variance_submitted","approval_task.assigned","approval_task.decided","invoice.variance_approved","invoice.ready","budget.committed","budget.actualized"]}</t>
+        </is>
+      </c>
+      <c r="AE11" t="n">
+        <v>5</v>
+      </c>
+      <c r="AF11" t="inlineStr">
+        <is>
+          <t>fin_ap2 เมนู ใบแจ้งหนี้ → บันทึกใบแจ้งหนี้ใหม่ → เลือก PO ของ H074 (SP0044) → เลือกไฟล์ใบแจ้งหนี้ที่สแกน → อัปโหลดและสร้างร่าง → กรอกเลขที่ S00829/A วันที่วันนี้ VAT ตามใบ → บันทึกหัวเอกสาร → แก้ราคาต่อหน่วยบรรทัด 1 เป็นราคาในใบ → บันทึกจำนวนและราคา → ยืนยันรหัสบัญชีทุกบรรทัด → ส่งจับคู่ → ไม่ตรง: ราคาสูงกว่า PO เกินเกณฑ์ ส่งถึงฝ่ายจัดซื้อ → proc_officer เมนู ใบสั่งซื้อ → ใบแจ้งหนี้ที่ไม่ตรงใบสั่งซื้อ → แถวเลขที่ผู้ขาย S00829/A → ขออนุมัติส่วนต่าง กรอกเหตุผล → ส่งขออนุมัติส่วนต่าง → dm_mep เปิดงาน ส่วนต่างราคาของใบแจ้งหนี้ (ข้อ IE-01) → อนุมัติ → ยืนยันอนุมัติ → fin_ap2 โหลดหน้าใบเดิม เห็นพร้อมจ่าย</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>S8</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>WHT</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>ใบค่าเช่ารถแบ็คโฮ หักภาษี ณ ที่จ่ายค่าเช่า 5% พร้อมยอดโอนคาดการณ์</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>fin_ap1</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>WEB</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>HIRE_SERVICE</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>CONI</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>P09-RENT</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>SITE-P09</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>SP0070</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>RNT-003</t>
+        </is>
+      </c>
+      <c r="O12" t="n">
+        <v>20</v>
+      </c>
+      <c r="P12" s="7" t="n">
+        <v>4608</v>
+      </c>
+      <c r="Q12" s="7" t="n">
+        <v>92160</v>
+      </c>
+      <c r="R12" s="7" t="n">
+        <v>6451.2</v>
+      </c>
+      <c r="S12" s="7" t="n">
+        <v>98611.2</v>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>H107</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>IV000893</t>
+        </is>
+      </c>
+      <c r="W12" s="7" t="n">
+        <v>4608</v>
+      </c>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="AD12" t="inlineStr">
+        <is>
+          <t>{"invoiceDate":"RUN_DATE","dueAfterDays":30,"file":"PDF","draft":{"channel":"UPLOAD","prefill":"MANUAL","defaultIncomeType":null},"poKind":"GOODS","acceptanceNeeded":false,"accountCode":"510301","costCenter":"CC-P09","whtIncomeType":"RENT","whtBp":500,"whtPickedInCoding":true,"whtRateConfirmed":false,"matchResult":"MATCHED","status":"READY_FOR_PAYMENT","payable":"98611.20","expectedWht":"4608.00","expectedTransfer":"94003.20","budget":{"committed":"-92160.00","actual":"92160.00","available":"0.00"},"whtCertificateAt":"PAYMENT_SCENE_11","events":["invoice.drafted","invoice.coding_confirmed","invoice.submitted","invoice.matched","invoice.ready","budget.actualized"]}</t>
+        </is>
+      </c>
+      <c r="AE12" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF12" t="inlineStr">
+        <is>
+          <t>fin_ap1 เมนู ใบแจ้งหนี้ → บันทึกใบแจ้งหนี้ใหม่ → เลือก PO ค่าเช่ารถแบ็คโฮของ H107 (SP0070) → เลือกไฟล์ → อัปโหลดและสร้างร่าง → กรอกเลขที่ IV000893 วันที่วันนี้ VAT ตามใบ → บันทึกหัวเอกสาร → ที่รหัสบัญชีบรรทัด 1 เลือกประเภทเงินได้ ค่าเช่าทรัพย์สิน 5% (ระบบยังไม่เลือกให้) → ยืนยันรหัสบัญชีทุกบรรทัด → ส่งจับคู่ → พร้อมจ่าย: ยอดที่ต้องจ่าย ภาษีหัก ณ ที่จ่ายคาดการณ์ 4,608.00 ยอดโอนคาดการณ์ 94,003.20 · หนังสือรับรอง 50 ทวิ ออกตอนจ่ายในฉาก 11</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>S9</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>PAYMENT_RUN</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>รอบจ่ายผู้ขาย 3 ราย ไฟล์แม่แบบกลาง และ 50 ทวิ ถึงอีเมลผู้ขาย</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>fin_tre1</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>fin_tre2 · cfo</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>WEB</t>
+        </is>
+      </c>
+      <c r="Q13" s="7" t="n">
+        <v>245560</v>
+      </c>
+      <c r="R13" s="7" t="n">
+        <v>17189.2</v>
+      </c>
+      <c r="S13" s="7" t="n">
+        <v>262749.2</v>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>PAID</t>
+        </is>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>PAY-01</t>
+        </is>
+      </c>
+      <c r="Z13" t="inlineStr">
+        <is>
+          <t>cfo</t>
+        </is>
+      </c>
+      <c r="AB13" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t>{"payer":"CB-01","parkFirst":"fin_tre2","docs":[{"scene":8,"supplier":"SP0029","payable":"100580.00","wht":"0.00","transfer":"100580.00"},{"scene":9,"supplier":"SP0044","payable":"63558.00","wht":"0.00","transfer":"63558.00"},{"scene":10,"supplier":"SP0070","payable":"98611.20","wht":"4608.00","transfer":"94003.20","whtIncomeType":"RENT","whtBp":500,"whtBase":"92160.00"}],"payable":"262749.20","wht":"4608.00","transfer":"258141.20","stepUp":true,"approveChannel":"LIFF","fileTemplate":"BCS-NEUTRAL-1","fileRows":3,"failed":[{"supplier":"SP0044","reasonTh":"บัญชีปิดแล้ว ธนาคารคืนเงิน"}],"paidTransfer":"194583.20","certificates":[{"supplier":"SP0070","form":"PND53","base":"92160.00","tax":"4608.00"}],"advices":["SP0029","SP0070"]}</t>
+        </is>
+      </c>
+      <c r="AE13" t="n">
+        <v>7</v>
+      </c>
+      <c r="AF13" t="inlineStr">
+        <is>
+          <t>fin_tre2: รอบจ่าย → เตรียมรอบจ่าย → สร้างร่างรอบจ่าย (รอบวันศุกร์ของใบที่ครบกำหนด เก็บไว้เป็นร่าง) · fin_tre1: รอบจ่าย → เตรียมรอบจ่าย (วันจ่ายศุกร์ถัดไป · CB-01 · ไม่มีใบครบกำหนดเหลือ) → สร้างร่างรอบจ่าย → เพิ่มใบแจ้งหนี้และเงินประกัน → ติ๊กใบของฉาก 8 9 10 (ป้าย จ่ายก่อนกำหนด) → เพิ่ม 3 เอกสารเข้ารอบ → ส่งขออนุมัติ · cfo: การ์ดใน LINE → อนุมัติ (ยืนยัน PIN) → ใส่ PIN → ยืนยันอนุมัติ · fin_tre1: แท็บไฟล์ → สร้างไฟล์ธนาคาร → ดาวน์โหลด BCS-NEUTRAL-1_NOT-A-BANK-FORMAT_… → ส่งธนาคารแล้ว → ยืนยันส่งธนาคารแล้ว · วันจ่าย: แท็บผลการจ่าย → SP0044 ไม่สำเร็จ (บัญชีปิดแล้ว ธนาคารคืนเงิน) → บันทึกผลการจ่าย → ยืนยันบันทึกผล · Mailpit: SP0029 และ SP0070 ได้อีเมลแจ้งการชำระ SP0070 แนบ 50 ทวิ ภ.ง.ด.53 · หน้า ภาษีหัก ณ ที่จ่าย มี 50 ทวิ ของ SP0070</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>12</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>S13</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>AI_QUOTE</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>โฟร์แมนแนบใบเสนอราคาเช่ารถแบ็คโฮ ให้ AI เติมฟอร์มและเสนอประเภท แล้วยืนยันทีละช่องก่อนส่ง</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>fm_p02</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>WEB</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>HIRE_SERVICE</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>CONB</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>P02-RENT</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>SITE-P02</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>SP0068</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>RNT-003</t>
+        </is>
+      </c>
+      <c r="O14" t="n">
+        <v>25</v>
+      </c>
+      <c r="P14" s="7" t="n">
+        <v>4848</v>
+      </c>
+      <c r="Q14" s="7" t="n">
+        <v>121200</v>
+      </c>
+      <c r="R14" s="7" t="n">
+        <v>8484</v>
+      </c>
+      <c r="S14" s="7" t="n">
+        <v>129684</v>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>DOC-049</t>
+        </is>
+      </c>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>ROUTED</t>
+        </is>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>PR-03</t>
+        </is>
+      </c>
+      <c r="Z14" t="inlineStr">
+        <is>
+          <t>ceo</t>
+        </is>
+      </c>
+      <c r="AB14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AD14" t="inlineStr">
+        <is>
+          <t>{"startType":"BUY_GOODS","aiType":"HIRE_SERVICE","finalType":"HIRE_SERVICE","uploadName":"QT-05317.pdf","intakeText":"เช่ารถแบ็คโฮตามใบเสนอราคาที่แนบ ใช้ที่หน้างานคอนโดบางนา","intakeRuns":2,"aiTitle":"ค่าเช่ารถแบ็คโฮ PC200 พร้อมผู้ควบคุม 25 วัน ตามใบเสนอราคา QT-05317","aiSite":"SITE-P02","aiSupplier":"SP0068","aiLines":[{"description":"ค่าเช่ารถแบ็คโฮ PC200 พร้อมผู้ควบคุม","qty":"25","unit":"วัน","unitPrice":"5187.36"}],"aiConfidence":96,"intakeMustConfirm":["lines.0.quantity","lines.0.unitPrice","suggestedSupplierId"],"priceIncludesVat":true,"form":{"scopeOfWork":"ค่าเช่ารถแบ็คโฮ PC200 พร้อมผู้ควบคุม ที่หน้างานโครงการ P02 คอนโดบางนา","servicePeriod":"25 วัน","processesPersonalData":"N","accessesSystems":"N","accessesPremises":"Y"},"serviceEndInDays":45,"quotation":{"docNo":"QT-05317","supplierName":"บริษัท พูนผลพาณิชย์เช่าเครื่องจักร จำกัด","amount":"129684.00","includesVat":true,"net":"121200.00","mustConfirm":["supplierId","amount"]},"singleSupplierReasonTh":"ผู้ขายรายนี้มีรถแบ็คโฮพร้อมผู้ควบคุมว่างตรงช่วงงานดินของโครงการ และเคยให้เช่าที่โครงการนี้ตามกำหนด","agentActions":{"INTAKE":"ACCEPTED","QUOTATION_READ":"ACCEPTED"},"flags":[],"pastOrderRef":"H053"}</t>
+        </is>
+      </c>
+      <c r="AE14" t="n">
+        <v>6</v>
+      </c>
+      <c r="AF14" t="inlineStr">
+        <is>
+          <t>fm_p02 เข้าเว็บ → ขอซื้อ/ขอจ้าง → ซื้อของ → กล่อง 'ให้ AI ช่วยกรอก (ไม่บังคับ)' แนบ QT-05317.pdf พิมพ์สั้น ๆ แล้วกด 'ให้ AI ช่วยกรอก' → เห็น 'ประเภทที่น่าจะตรงกว่า: จ้างบริการ' กด 'เปลี่ยนประเภท' → ในฟอร์มจ้างบริการแนบไฟล์เดิมแล้วกด 'ให้ AI ช่วยกรอก' อีกครั้ง → ค่าที่เติมมีป้าย 'เติมโดย AI โปรดตรวจ' ติ๊กยืนยันจำนวน ราคาต่อหน่วย และผู้ขายที่แนะนำทีละช่อง แล้วกด 'ยืนยันค่าที่เหลือทั้งหมด' → กรอกขอบเขตงานและระยะเวลา → ขั้นรายการ เลือกบรรทัดงบ P02-RENT ติ๊ก 'ราคาที่กรอกรวม VAT แล้ว' ใส่วันสิ้นสุดบริการ → ขั้นผู้ขาย 'เพิ่มใบเสนอราคา' แนบไฟล์ กด 'อ่านใบเสนอราคาที่ 1 จากไฟล์' ยืนยันผู้ขายและยอดทีละช่อง ติ๊ก 'เลือกใช้ใบเสนอราคาที่ 1' → ตอบคำถามคัดกรอง 3 ข้อ → ขั้นเอกสาร กรอก 'เหตุผลกรณีมีผู้ขายรายเดียว' → ตรวจและส่ง กด 'ส่งขออนุมัติ' → เห็น 'ส่งขออนุมัติแล้ว รอ ปิยะนุช สุขประเสริฐ พิจารณา'</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>S13</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>AI_BRIEF</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>กรรมการผู้จัดการเปิดงานอนุมัติค่าเช่ารถแบ็คโฮ เห็นสรุปจาก AI ที่ตัวเลขทุกตัวมาจากระบบ</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>ceo</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>WEB</t>
+        </is>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Y15" t="inlineStr">
+        <is>
+          <t>PR-03</t>
+        </is>
+      </c>
+      <c r="Z15" t="inlineStr">
+        <is>
+          <t>ceo</t>
+        </is>
+      </c>
+      <c r="AB15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AD15" t="inlineStr">
+        <is>
+          <t>{"requestOfScene":12,"briefSentences":["คำขอนี้ยอด {{v:amount}} บาท ตามข้อ {{v:doaRule}}","งบคงเหลือหลังคำขอนี้ {{v:budgetRemaining}} บาท","มีใบเสนอราคา {{v:quoteCount}} ใบ"],"facts":{"amount":"129684.00","amountBasis":"GROSS","doaRule":"PR-03","quoteCount":1,"quoteChosenLowest":"YES","priceReference":"NONE","slaOverdue":"NO"},"factsFromDb":["supplierPoCount","supplierLastPoAmount","slaHoursLeft"],"supplierPoCountFromHistory":4,"boxButtons":0,"reasonOutsideBox":true,"decide":false}</t>
+        </is>
+      </c>
+      <c r="AE15" t="n">
+        <v>2</v>
+      </c>
+      <c r="AF15" t="inlineStr">
+        <is>
+          <t>ceo เข้าเว็บ (รหัสผ่าน + รหัส 6 หลัก) → งานของฉัน → เปิดงานของคำขอค่าเช่ารถแบ็คโฮ → ชี้กล่อง 'สรุปจาก AI': ยอดตามฐาน DOA ข้อ PR-03 งบคงเหลือหลังคำขอ และจำนวนใบเสนอราคา พร้อม 'AI อาจผิดพลาด ตรวจกับเอกสาร' → ชี้ว่าในกล่องไม่มีปุ่มตัดสิน และเหตุผลกรณีมีผู้ขายรายเดียวอยู่ในรายละเอียดคำขอด้านล่าง (ฉากนี้ยังไม่กดอนุมัติ)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>14</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>S13</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>ASK_AI</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>ถาม BCS AI ว่างบไหนใกล้หมด และคนที่ไม่มีสิทธิ์ได้คำตอบว่าไม่พบข้อมูลในสิทธิ์</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>ceo</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>se_p01a</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>WEB</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>MKT</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>MKT-OPEX</t>
+        </is>
+      </c>
+      <c r="X16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AB16" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AD16" t="inlineStr">
+        <is>
+          <t>{"questionTh":"งบไหนใกล้หมด","plannedTools":["budget_status"],"expectedBudgetKeys":["MKT-OPEX"],"firstRowKey":"MKT-OPEX","lowPct":10,"fixtureKind":"TABLE","liveKind":"ANSWER","linkPrefix":"/budgets/","deniedMember":"se_p01a","deniedKind":"NOT_FOUND"}</t>
+        </is>
+      </c>
+      <c r="AE16" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF16" t="inlineStr">
+        <is>
+          <t>ceo กดปุ่มค้นหา (⌘K) พิมพ์ 'งบไหนใกล้หมด' → เลือก 'ถาม BCS AI: งบไหนใกล้หมด' → คำตอบแสดง MKT-OPEX งบคงเหลือต่ำกว่า 10% อยู่บรรทัดแรก พร้อมปุ่ม 'เปิด' ไปหน้าบรรทัดงบ (วัน demo ที่ AI จริงจะตอบเป็นประโยค) → se_p01a เข้าเว็บ ถามคำเดียวกัน → 'ไม่พบข้อมูลในสิทธิ์ของคุณ'</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>S17</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>CHAT_REQUEST</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>ขอซื้อเหล็กผ่านแชท LINE ด้วยรูปใบเสนอราคา ให้ AI ร่างแล้วยืนยันใน LIFF</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>se_p01a</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>LINE_CHAT</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>BUY_GOODS</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>CONB</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>P01-MAT</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>SITE-P01</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>SP0030</t>
+        </is>
+      </c>
+      <c r="O17" t="n">
+        <v>1</v>
+      </c>
+      <c r="P17" s="7" t="n">
+        <v>24411</v>
+      </c>
+      <c r="Q17" s="7" t="n">
+        <v>24411</v>
+      </c>
+      <c r="R17" s="7" t="n">
+        <v>1708.77</v>
+      </c>
+      <c r="S17" s="7" t="n">
+        <v>26119.77</v>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>DOC-031</t>
+        </is>
+      </c>
+      <c r="X17" t="inlineStr">
+        <is>
+          <t>ROUTED</t>
+        </is>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>PR-02</t>
+        </is>
+      </c>
+      <c r="Z17" t="inlineStr">
+        <is>
+          <t>vp_ops</t>
+        </is>
+      </c>
+      <c r="AB17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AD17" t="inlineStr">
+        <is>
+          <t>{"chatText":"ขอซื้อเหล็กข้ออ้อย DB25 1 ตัน ส่งไซต์พระราม 9","photos":1,"aiType":"BUY_GOODS","line":{"description":"เหล็กข้ออ้อย DB25 SD40","unit":"ตัน"},"mustConfirm":["lines.0.quantity","lines.0.unitPrice"],"attachments":["OTHER"],"submitChannel":"LIFF","approverCard":true}</t>
+        </is>
+      </c>
+      <c r="AE17" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF17" t="inlineStr">
+        <is>
+          <t>se_p01a ในแชท LINE ของบริษัท: พิมพ์ข้อความตามแถว แล้วส่งรูปใบเสนอราคา (DOC-031) → แตะปุ่ม "ตรวจและส่งคำขอ" → LIFF: เห็น "AI กำลังอ่านข้อความและรูป" แล้วค่าที่ AI อ่านมีป้าย "เติมโดย AI โปรดตรวจ" ประเภท ซื้อของ ถูกเลือกไว้ → "สร้างร่างคำขอ" → ในกล่อง "ค่าที่ AI เติมรอยืนยัน" ติ๊กทีละช่อง (จำนวน ราคาต่อหน่วย ผู้ขาย ฯลฯ) → "ยืนยันค่าที่ตรวจแล้ว" → เลือกบรรทัดงบ P01-MAT ของปีงบนี้ → "ไปขั้นถัดไป: รายการที่ขอ" ตรวจยอดก่อน VAT VAT และรวม → "ไปขั้นถัดไป: ตรวจและส่ง" เห็นเส้นทางไปรองกรรมการผู้จัดการสายปฏิบัติการ (ข้อ PR-02) → "ส่งขออนุมัติ" · vp_ops ได้การ์ดงานใน LINE · ถ้าถูกถามว่าปิด AI ได้ไหม: ผู้ดูแลปิดโมดูล AI แล้วทำซ้ำได้ครบ (พิสูจน์แล้วใน e2e @s17 ฉาก 6)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>16</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>S13</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>AI_INVOICE</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>AI อ่านใบแจ้งหนี้ปูนซีเมนต์ให้การเงิน ยืนยันทีละช่องก่อนส่งจับคู่</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>fin_ap1</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>WEB</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>BUY_GOODS</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>CONI</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>P06-MAT</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>SITE-P06</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>SP0018</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>MAT-001</t>
+        </is>
+      </c>
+      <c r="O18" t="n">
+        <v>33</v>
+      </c>
+      <c r="P18" s="7" t="n">
+        <v>145</v>
+      </c>
+      <c r="Q18" s="7" t="n">
+        <v>4785</v>
+      </c>
+      <c r="R18" s="7" t="n">
+        <v>334.95</v>
+      </c>
+      <c r="S18" s="7" t="n">
+        <v>5119.95</v>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>H188</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>บก.000767</t>
+        </is>
+      </c>
+      <c r="W18" s="7" t="n">
+        <v>145</v>
+      </c>
+      <c r="X18" t="inlineStr">
+        <is>
+          <t>MATCHED</t>
+        </is>
+      </c>
+      <c r="AD18" t="inlineStr">
+        <is>
+          <t>{"aiPurpose":"INVOICE_READ","aiAnswer":"SCENE_FROM_SHEET","reading":{"docType":"TAX_INVOICE","docNo":"บก.000767","docDate":"RUN_DATE","priceIncludesVat":false,"lines":[{"itemCode":"MAT-001","qty":"33","unitPrice":"145.00","amount":"4785.00"}],"net":"4785.00","vat":"334.95","gross":"5119.95"},"invoiceDate":"RUN_DATE","dueAfterDays":45,"draft":{"channel":"UPLOAD"},"agentAction":{"status":"ACCEPTED","subjectType":"INVOICE"},"accountCode":"510101","costCenter":"CC-P06","matchResult":"MATCHED","status":"READY_FOR_PAYMENT","payable":"5119.95","expectedWht":"0.00","budget":{"committed":"-4785.00","actual":"4785.00","available":"0.00"}}</t>
+        </is>
+      </c>
+      <c r="AE18" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF18" t="inlineStr">
+        <is>
+          <t>fin_ap1 เมนู ใบแจ้งหนี้ → บันทึกใบแจ้งหนี้ใหม่ → เลือก PO ปูนซีเมนต์ของ H188 (SP0018) → เลือกรูปใบแจ้งหนี้ → อ่านไฟล์ด้วย AI → รอ AI อ่าน → ร่างเปิดพร้อมกล่อง ค่าที่ AI อ่านจากใบแจ้งหนี้ ป้าย เติมโดย AI โปรดตรวจ → ยืนยันรหัสบัญชีทุกบรรทัด → ลองส่งจับคู่ ระบบไม่ให้ส่งจนยืนยันครบ → ติ๊กยืนยันทีละช่องเทียบกับไฟล์ → บันทึกการยืนยัน → ส่งจับคู่ → พร้อมจ่าย</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>